<commit_message>
Log Oct 3 count and reviews (pharmacy 9)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01RnF4y3zxCG7NcjFkMnYdwu
</commit_message>
<xml_diff>
--- a/inventory/jard_log.xlsx
+++ b/inventory/jard_log.xlsx
@@ -10,7 +10,7 @@
     <sheet name="السجل" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'السجل'!$A$1:$I$57</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'السجل'!$A$1:$I$62</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -468,7 +468,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I58"/>
+  <dimension ref="A1:I63"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -2770,25 +2770,224 @@
       </c>
     </row>
     <row r="58">
-      <c r="A58" s="4" t="inlineStr">
+      <c r="A58" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-03</t>
+        </is>
+      </c>
+      <c r="B58" s="2" t="inlineStr">
+        <is>
+          <t>السبت</t>
+        </is>
+      </c>
+      <c r="C58" s="2" t="inlineStr">
+        <is>
+          <t>الدلم</t>
+        </is>
+      </c>
+      <c r="D58" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="E58" s="2" t="inlineStr">
+        <is>
+          <t>د. علي خليفة</t>
+        </is>
+      </c>
+      <c r="F58" s="2" t="inlineStr">
+        <is>
+          <t>نعم</t>
+        </is>
+      </c>
+      <c r="G58" s="2" t="inlineStr">
+        <is>
+          <t>نعم</t>
+        </is>
+      </c>
+      <c r="H58" s="2" t="inlineStr">
+        <is>
+          <t>جرد + مراجعة</t>
+        </is>
+      </c>
+      <c r="I58" s="3" t="n">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-03</t>
+        </is>
+      </c>
+      <c r="B59" s="2" t="inlineStr">
+        <is>
+          <t>السبت</t>
+        </is>
+      </c>
+      <c r="C59" s="2" t="inlineStr">
+        <is>
+          <t>الدلم</t>
+        </is>
+      </c>
+      <c r="D59" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="E59" s="2" t="inlineStr">
+        <is>
+          <t>د. حسام شلش</t>
+        </is>
+      </c>
+      <c r="F59" s="2" t="inlineStr"/>
+      <c r="G59" s="2" t="inlineStr">
+        <is>
+          <t>نعم</t>
+        </is>
+      </c>
+      <c r="H59" s="2" t="inlineStr">
+        <is>
+          <t>مراجعة فقط</t>
+        </is>
+      </c>
+      <c r="I59" s="3" t="n">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-03</t>
+        </is>
+      </c>
+      <c r="B60" s="2" t="inlineStr">
+        <is>
+          <t>السبت</t>
+        </is>
+      </c>
+      <c r="C60" s="2" t="inlineStr">
+        <is>
+          <t>الدلم</t>
+        </is>
+      </c>
+      <c r="D60" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="E60" s="2" t="inlineStr">
+        <is>
+          <t>د. السيد حسن</t>
+        </is>
+      </c>
+      <c r="F60" s="2" t="inlineStr"/>
+      <c r="G60" s="2" t="inlineStr">
+        <is>
+          <t>نعم</t>
+        </is>
+      </c>
+      <c r="H60" s="2" t="inlineStr">
+        <is>
+          <t>مراجعة فقط</t>
+        </is>
+      </c>
+      <c r="I60" s="3" t="n">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-03</t>
+        </is>
+      </c>
+      <c r="B61" s="2" t="inlineStr">
+        <is>
+          <t>السبت</t>
+        </is>
+      </c>
+      <c r="C61" s="2" t="inlineStr">
+        <is>
+          <t>الدلم</t>
+        </is>
+      </c>
+      <c r="D61" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="E61" s="2" t="inlineStr">
+        <is>
+          <t>د. أيمن حسين</t>
+        </is>
+      </c>
+      <c r="F61" s="2" t="inlineStr"/>
+      <c r="G61" s="2" t="inlineStr">
+        <is>
+          <t>نعم</t>
+        </is>
+      </c>
+      <c r="H61" s="2" t="inlineStr">
+        <is>
+          <t>مراجعة فقط</t>
+        </is>
+      </c>
+      <c r="I61" s="3" t="n">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-03</t>
+        </is>
+      </c>
+      <c r="B62" s="2" t="inlineStr">
+        <is>
+          <t>السبت</t>
+        </is>
+      </c>
+      <c r="C62" s="2" t="inlineStr">
+        <is>
+          <t>الدلم</t>
+        </is>
+      </c>
+      <c r="D62" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="E62" s="2" t="inlineStr">
+        <is>
+          <t>د. الحسن الغنيمي</t>
+        </is>
+      </c>
+      <c r="F62" s="2" t="inlineStr"/>
+      <c r="G62" s="2" t="inlineStr">
+        <is>
+          <t>نعم</t>
+        </is>
+      </c>
+      <c r="H62" s="2" t="inlineStr">
+        <is>
+          <t>مراجعة فقط</t>
+        </is>
+      </c>
+      <c r="I62" s="3" t="n">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="4" t="inlineStr">
         <is>
           <t>الإجمالي</t>
         </is>
       </c>
-      <c r="B58" s="4" t="n"/>
-      <c r="C58" s="4" t="n"/>
-      <c r="D58" s="4" t="n"/>
-      <c r="E58" s="4" t="n"/>
-      <c r="F58" s="4" t="n"/>
-      <c r="G58" s="4" t="n"/>
-      <c r="H58" s="4" t="n"/>
-      <c r="I58" s="5">
-        <f>SUM(I2:I57)</f>
-        <v>9100</v>
+      <c r="B63" s="4" t="n"/>
+      <c r="C63" s="4" t="n"/>
+      <c r="D63" s="4" t="n"/>
+      <c r="E63" s="4" t="n"/>
+      <c r="F63" s="4" t="n"/>
+      <c r="G63" s="4" t="n"/>
+      <c r="H63" s="4" t="n"/>
+      <c r="I63" s="5">
+        <f>SUM(I2:I62)</f>
+        <v>9900</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:I57"/>
+  <autoFilter ref="A1:I62"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Log Oct 4 counts and reviews (pharmacies 32 and 39)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01RnF4y3zxCG7NcjFkMnYdwu
</commit_message>
<xml_diff>
--- a/inventory/jard_log.xlsx
+++ b/inventory/jard_log.xlsx
@@ -10,7 +10,7 @@
     <sheet name="السجل" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'السجل'!$A$1:$I$62</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'السجل'!$A$1:$I$70</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -468,7 +468,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I63"/>
+  <dimension ref="A1:I71"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -2969,25 +2969,345 @@
       </c>
     </row>
     <row r="63">
-      <c r="A63" s="4" t="inlineStr">
+      <c r="A63" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-04</t>
+        </is>
+      </c>
+      <c r="B63" s="2" t="inlineStr">
+        <is>
+          <t>الأحد</t>
+        </is>
+      </c>
+      <c r="C63" s="2" t="inlineStr">
+        <is>
+          <t>الحوطة</t>
+        </is>
+      </c>
+      <c r="D63" s="2" t="n">
+        <v>32</v>
+      </c>
+      <c r="E63" s="2" t="inlineStr">
+        <is>
+          <t>د. حسام شلش</t>
+        </is>
+      </c>
+      <c r="F63" s="2" t="inlineStr">
+        <is>
+          <t>نعم</t>
+        </is>
+      </c>
+      <c r="G63" s="2" t="inlineStr">
+        <is>
+          <t>نعم</t>
+        </is>
+      </c>
+      <c r="H63" s="2" t="inlineStr">
+        <is>
+          <t>جرد + مراجعة</t>
+        </is>
+      </c>
+      <c r="I63" s="3" t="n">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-04</t>
+        </is>
+      </c>
+      <c r="B64" s="2" t="inlineStr">
+        <is>
+          <t>الأحد</t>
+        </is>
+      </c>
+      <c r="C64" s="2" t="inlineStr">
+        <is>
+          <t>الحوطة</t>
+        </is>
+      </c>
+      <c r="D64" s="2" t="n">
+        <v>32</v>
+      </c>
+      <c r="E64" s="2" t="inlineStr">
+        <is>
+          <t>د. السيد حسن</t>
+        </is>
+      </c>
+      <c r="F64" s="2" t="inlineStr"/>
+      <c r="G64" s="2" t="inlineStr">
+        <is>
+          <t>نعم</t>
+        </is>
+      </c>
+      <c r="H64" s="2" t="inlineStr">
+        <is>
+          <t>مراجعة فقط</t>
+        </is>
+      </c>
+      <c r="I64" s="3" t="n">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-04</t>
+        </is>
+      </c>
+      <c r="B65" s="2" t="inlineStr">
+        <is>
+          <t>الأحد</t>
+        </is>
+      </c>
+      <c r="C65" s="2" t="inlineStr">
+        <is>
+          <t>الحوطة</t>
+        </is>
+      </c>
+      <c r="D65" s="2" t="n">
+        <v>32</v>
+      </c>
+      <c r="E65" s="2" t="inlineStr">
+        <is>
+          <t>د. الحسن الغنيمي</t>
+        </is>
+      </c>
+      <c r="F65" s="2" t="inlineStr"/>
+      <c r="G65" s="2" t="inlineStr">
+        <is>
+          <t>نعم</t>
+        </is>
+      </c>
+      <c r="H65" s="2" t="inlineStr">
+        <is>
+          <t>مراجعة فقط</t>
+        </is>
+      </c>
+      <c r="I65" s="3" t="n">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-04</t>
+        </is>
+      </c>
+      <c r="B66" s="2" t="inlineStr">
+        <is>
+          <t>الأحد</t>
+        </is>
+      </c>
+      <c r="C66" s="2" t="inlineStr">
+        <is>
+          <t>الحوطة</t>
+        </is>
+      </c>
+      <c r="D66" s="2" t="n">
+        <v>32</v>
+      </c>
+      <c r="E66" s="2" t="inlineStr">
+        <is>
+          <t>د. محمد جمال</t>
+        </is>
+      </c>
+      <c r="F66" s="2" t="inlineStr"/>
+      <c r="G66" s="2" t="inlineStr">
+        <is>
+          <t>نعم</t>
+        </is>
+      </c>
+      <c r="H66" s="2" t="inlineStr">
+        <is>
+          <t>مراجعة فقط</t>
+        </is>
+      </c>
+      <c r="I66" s="3" t="n">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-04</t>
+        </is>
+      </c>
+      <c r="B67" s="2" t="inlineStr">
+        <is>
+          <t>الأحد</t>
+        </is>
+      </c>
+      <c r="C67" s="2" t="inlineStr">
+        <is>
+          <t>الحوطة</t>
+        </is>
+      </c>
+      <c r="D67" s="2" t="n">
+        <v>39</v>
+      </c>
+      <c r="E67" s="2" t="inlineStr">
+        <is>
+          <t>د. حسام شلش</t>
+        </is>
+      </c>
+      <c r="F67" s="2" t="inlineStr">
+        <is>
+          <t>نعم</t>
+        </is>
+      </c>
+      <c r="G67" s="2" t="inlineStr">
+        <is>
+          <t>نعم</t>
+        </is>
+      </c>
+      <c r="H67" s="2" t="inlineStr">
+        <is>
+          <t>جرد + مراجعة</t>
+        </is>
+      </c>
+      <c r="I67" s="3" t="n">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-04</t>
+        </is>
+      </c>
+      <c r="B68" s="2" t="inlineStr">
+        <is>
+          <t>الأحد</t>
+        </is>
+      </c>
+      <c r="C68" s="2" t="inlineStr">
+        <is>
+          <t>الحوطة</t>
+        </is>
+      </c>
+      <c r="D68" s="2" t="n">
+        <v>39</v>
+      </c>
+      <c r="E68" s="2" t="inlineStr">
+        <is>
+          <t>د. السيد حسن</t>
+        </is>
+      </c>
+      <c r="F68" s="2" t="inlineStr"/>
+      <c r="G68" s="2" t="inlineStr">
+        <is>
+          <t>نعم</t>
+        </is>
+      </c>
+      <c r="H68" s="2" t="inlineStr">
+        <is>
+          <t>مراجعة فقط</t>
+        </is>
+      </c>
+      <c r="I68" s="3" t="n">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-04</t>
+        </is>
+      </c>
+      <c r="B69" s="2" t="inlineStr">
+        <is>
+          <t>الأحد</t>
+        </is>
+      </c>
+      <c r="C69" s="2" t="inlineStr">
+        <is>
+          <t>الحوطة</t>
+        </is>
+      </c>
+      <c r="D69" s="2" t="n">
+        <v>39</v>
+      </c>
+      <c r="E69" s="2" t="inlineStr">
+        <is>
+          <t>د. الحسن الغنيمي</t>
+        </is>
+      </c>
+      <c r="F69" s="2" t="inlineStr"/>
+      <c r="G69" s="2" t="inlineStr">
+        <is>
+          <t>نعم</t>
+        </is>
+      </c>
+      <c r="H69" s="2" t="inlineStr">
+        <is>
+          <t>مراجعة فقط</t>
+        </is>
+      </c>
+      <c r="I69" s="3" t="n">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-04</t>
+        </is>
+      </c>
+      <c r="B70" s="2" t="inlineStr">
+        <is>
+          <t>الأحد</t>
+        </is>
+      </c>
+      <c r="C70" s="2" t="inlineStr">
+        <is>
+          <t>الحوطة</t>
+        </is>
+      </c>
+      <c r="D70" s="2" t="n">
+        <v>39</v>
+      </c>
+      <c r="E70" s="2" t="inlineStr">
+        <is>
+          <t>د. محمد جمال</t>
+        </is>
+      </c>
+      <c r="F70" s="2" t="inlineStr"/>
+      <c r="G70" s="2" t="inlineStr">
+        <is>
+          <t>نعم</t>
+        </is>
+      </c>
+      <c r="H70" s="2" t="inlineStr">
+        <is>
+          <t>مراجعة فقط</t>
+        </is>
+      </c>
+      <c r="I70" s="3" t="n">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="4" t="inlineStr">
         <is>
           <t>الإجمالي</t>
         </is>
       </c>
-      <c r="B63" s="4" t="n"/>
-      <c r="C63" s="4" t="n"/>
-      <c r="D63" s="4" t="n"/>
-      <c r="E63" s="4" t="n"/>
-      <c r="F63" s="4" t="n"/>
-      <c r="G63" s="4" t="n"/>
-      <c r="H63" s="4" t="n"/>
-      <c r="I63" s="5">
-        <f>SUM(I2:I62)</f>
-        <v>9900</v>
+      <c r="B71" s="4" t="n"/>
+      <c r="C71" s="4" t="n"/>
+      <c r="D71" s="4" t="n"/>
+      <c r="E71" s="4" t="n"/>
+      <c r="F71" s="4" t="n"/>
+      <c r="G71" s="4" t="n"/>
+      <c r="H71" s="4" t="n"/>
+      <c r="I71" s="5">
+        <f>SUM(I2:I70)</f>
+        <v>11200</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:I62"/>
+  <autoFilter ref="A1:I70"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Log Oct 5 counts and reviews (pharmacies 33 and 34)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01RnF4y3zxCG7NcjFkMnYdwu
</commit_message>
<xml_diff>
--- a/inventory/jard_log.xlsx
+++ b/inventory/jard_log.xlsx
@@ -10,7 +10,7 @@
     <sheet name="السجل" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'السجل'!$A$1:$I$70</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'السجل'!$A$1:$I$78</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -468,7 +468,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I71"/>
+  <dimension ref="A1:I79"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -3289,25 +3289,345 @@
       </c>
     </row>
     <row r="71">
-      <c r="A71" s="4" t="inlineStr">
+      <c r="A71" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+      <c r="B71" s="2" t="inlineStr">
+        <is>
+          <t>الاثنين</t>
+        </is>
+      </c>
+      <c r="C71" s="2" t="inlineStr">
+        <is>
+          <t>الأفلاج</t>
+        </is>
+      </c>
+      <c r="D71" s="2" t="n">
+        <v>33</v>
+      </c>
+      <c r="E71" s="2" t="inlineStr">
+        <is>
+          <t>د. السيد حسن</t>
+        </is>
+      </c>
+      <c r="F71" s="2" t="inlineStr">
+        <is>
+          <t>نعم</t>
+        </is>
+      </c>
+      <c r="G71" s="2" t="inlineStr">
+        <is>
+          <t>نعم</t>
+        </is>
+      </c>
+      <c r="H71" s="2" t="inlineStr">
+        <is>
+          <t>جرد + مراجعة</t>
+        </is>
+      </c>
+      <c r="I71" s="3" t="n">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+      <c r="B72" s="2" t="inlineStr">
+        <is>
+          <t>الاثنين</t>
+        </is>
+      </c>
+      <c r="C72" s="2" t="inlineStr">
+        <is>
+          <t>الأفلاج</t>
+        </is>
+      </c>
+      <c r="D72" s="2" t="n">
+        <v>33</v>
+      </c>
+      <c r="E72" s="2" t="inlineStr">
+        <is>
+          <t>د. حسام شلش</t>
+        </is>
+      </c>
+      <c r="F72" s="2" t="inlineStr"/>
+      <c r="G72" s="2" t="inlineStr">
+        <is>
+          <t>نعم</t>
+        </is>
+      </c>
+      <c r="H72" s="2" t="inlineStr">
+        <is>
+          <t>مراجعة فقط</t>
+        </is>
+      </c>
+      <c r="I72" s="3" t="n">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+      <c r="B73" s="2" t="inlineStr">
+        <is>
+          <t>الاثنين</t>
+        </is>
+      </c>
+      <c r="C73" s="2" t="inlineStr">
+        <is>
+          <t>الأفلاج</t>
+        </is>
+      </c>
+      <c r="D73" s="2" t="n">
+        <v>33</v>
+      </c>
+      <c r="E73" s="2" t="inlineStr">
+        <is>
+          <t>د. الحسن الغنيمي</t>
+        </is>
+      </c>
+      <c r="F73" s="2" t="inlineStr"/>
+      <c r="G73" s="2" t="inlineStr">
+        <is>
+          <t>نعم</t>
+        </is>
+      </c>
+      <c r="H73" s="2" t="inlineStr">
+        <is>
+          <t>مراجعة فقط</t>
+        </is>
+      </c>
+      <c r="I73" s="3" t="n">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+      <c r="B74" s="2" t="inlineStr">
+        <is>
+          <t>الاثنين</t>
+        </is>
+      </c>
+      <c r="C74" s="2" t="inlineStr">
+        <is>
+          <t>الأفلاج</t>
+        </is>
+      </c>
+      <c r="D74" s="2" t="n">
+        <v>33</v>
+      </c>
+      <c r="E74" s="2" t="inlineStr">
+        <is>
+          <t>د. محمد جمال</t>
+        </is>
+      </c>
+      <c r="F74" s="2" t="inlineStr"/>
+      <c r="G74" s="2" t="inlineStr">
+        <is>
+          <t>نعم</t>
+        </is>
+      </c>
+      <c r="H74" s="2" t="inlineStr">
+        <is>
+          <t>مراجعة فقط</t>
+        </is>
+      </c>
+      <c r="I74" s="3" t="n">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+      <c r="B75" s="2" t="inlineStr">
+        <is>
+          <t>الاثنين</t>
+        </is>
+      </c>
+      <c r="C75" s="2" t="inlineStr">
+        <is>
+          <t>الأفلاج</t>
+        </is>
+      </c>
+      <c r="D75" s="2" t="n">
+        <v>34</v>
+      </c>
+      <c r="E75" s="2" t="inlineStr">
+        <is>
+          <t>د. السيد حسن</t>
+        </is>
+      </c>
+      <c r="F75" s="2" t="inlineStr">
+        <is>
+          <t>نعم</t>
+        </is>
+      </c>
+      <c r="G75" s="2" t="inlineStr">
+        <is>
+          <t>نعم</t>
+        </is>
+      </c>
+      <c r="H75" s="2" t="inlineStr">
+        <is>
+          <t>جرد + مراجعة</t>
+        </is>
+      </c>
+      <c r="I75" s="3" t="n">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+      <c r="B76" s="2" t="inlineStr">
+        <is>
+          <t>الاثنين</t>
+        </is>
+      </c>
+      <c r="C76" s="2" t="inlineStr">
+        <is>
+          <t>الأفلاج</t>
+        </is>
+      </c>
+      <c r="D76" s="2" t="n">
+        <v>34</v>
+      </c>
+      <c r="E76" s="2" t="inlineStr">
+        <is>
+          <t>د. حسام شلش</t>
+        </is>
+      </c>
+      <c r="F76" s="2" t="inlineStr"/>
+      <c r="G76" s="2" t="inlineStr">
+        <is>
+          <t>نعم</t>
+        </is>
+      </c>
+      <c r="H76" s="2" t="inlineStr">
+        <is>
+          <t>مراجعة فقط</t>
+        </is>
+      </c>
+      <c r="I76" s="3" t="n">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+      <c r="B77" s="2" t="inlineStr">
+        <is>
+          <t>الاثنين</t>
+        </is>
+      </c>
+      <c r="C77" s="2" t="inlineStr">
+        <is>
+          <t>الأفلاج</t>
+        </is>
+      </c>
+      <c r="D77" s="2" t="n">
+        <v>34</v>
+      </c>
+      <c r="E77" s="2" t="inlineStr">
+        <is>
+          <t>د. الحسن الغنيمي</t>
+        </is>
+      </c>
+      <c r="F77" s="2" t="inlineStr"/>
+      <c r="G77" s="2" t="inlineStr">
+        <is>
+          <t>نعم</t>
+        </is>
+      </c>
+      <c r="H77" s="2" t="inlineStr">
+        <is>
+          <t>مراجعة فقط</t>
+        </is>
+      </c>
+      <c r="I77" s="3" t="n">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+      <c r="B78" s="2" t="inlineStr">
+        <is>
+          <t>الاثنين</t>
+        </is>
+      </c>
+      <c r="C78" s="2" t="inlineStr">
+        <is>
+          <t>الأفلاج</t>
+        </is>
+      </c>
+      <c r="D78" s="2" t="n">
+        <v>34</v>
+      </c>
+      <c r="E78" s="2" t="inlineStr">
+        <is>
+          <t>د. محمد جمال</t>
+        </is>
+      </c>
+      <c r="F78" s="2" t="inlineStr"/>
+      <c r="G78" s="2" t="inlineStr">
+        <is>
+          <t>نعم</t>
+        </is>
+      </c>
+      <c r="H78" s="2" t="inlineStr">
+        <is>
+          <t>مراجعة فقط</t>
+        </is>
+      </c>
+      <c r="I78" s="3" t="n">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="4" t="inlineStr">
         <is>
           <t>الإجمالي</t>
         </is>
       </c>
-      <c r="B71" s="4" t="n"/>
-      <c r="C71" s="4" t="n"/>
-      <c r="D71" s="4" t="n"/>
-      <c r="E71" s="4" t="n"/>
-      <c r="F71" s="4" t="n"/>
-      <c r="G71" s="4" t="n"/>
-      <c r="H71" s="4" t="n"/>
-      <c r="I71" s="5">
-        <f>SUM(I2:I70)</f>
-        <v>11200</v>
+      <c r="B79" s="4" t="n"/>
+      <c r="C79" s="4" t="n"/>
+      <c r="D79" s="4" t="n"/>
+      <c r="E79" s="4" t="n"/>
+      <c r="F79" s="4" t="n"/>
+      <c r="G79" s="4" t="n"/>
+      <c r="H79" s="4" t="n"/>
+      <c r="I79" s="5">
+        <f>SUM(I2:I78)</f>
+        <v>12500</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:I70"/>
+  <autoFilter ref="A1:I78"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Log Oct 6 counts and reviews (pharmacies 35 and 53)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01RnF4y3zxCG7NcjFkMnYdwu
</commit_message>
<xml_diff>
--- a/inventory/jard_log.xlsx
+++ b/inventory/jard_log.xlsx
@@ -10,7 +10,7 @@
     <sheet name="السجل" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'السجل'!$A$1:$I$78</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'السجل'!$A$1:$I$86</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -468,7 +468,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I79"/>
+  <dimension ref="A1:I87"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -3609,25 +3609,345 @@
       </c>
     </row>
     <row r="79">
-      <c r="A79" s="4" t="inlineStr">
+      <c r="A79" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="B79" s="2" t="inlineStr">
+        <is>
+          <t>الثلاثاء</t>
+        </is>
+      </c>
+      <c r="C79" s="2" t="inlineStr">
+        <is>
+          <t>السليل</t>
+        </is>
+      </c>
+      <c r="D79" s="2" t="n">
+        <v>35</v>
+      </c>
+      <c r="E79" s="2" t="inlineStr">
+        <is>
+          <t>د. حسام شلش</t>
+        </is>
+      </c>
+      <c r="F79" s="2" t="inlineStr">
+        <is>
+          <t>نعم</t>
+        </is>
+      </c>
+      <c r="G79" s="2" t="inlineStr">
+        <is>
+          <t>نعم</t>
+        </is>
+      </c>
+      <c r="H79" s="2" t="inlineStr">
+        <is>
+          <t>جرد + مراجعة</t>
+        </is>
+      </c>
+      <c r="I79" s="3" t="n">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="B80" s="2" t="inlineStr">
+        <is>
+          <t>الثلاثاء</t>
+        </is>
+      </c>
+      <c r="C80" s="2" t="inlineStr">
+        <is>
+          <t>السليل</t>
+        </is>
+      </c>
+      <c r="D80" s="2" t="n">
+        <v>35</v>
+      </c>
+      <c r="E80" s="2" t="inlineStr">
+        <is>
+          <t>د. السيد حسن</t>
+        </is>
+      </c>
+      <c r="F80" s="2" t="inlineStr"/>
+      <c r="G80" s="2" t="inlineStr">
+        <is>
+          <t>نعم</t>
+        </is>
+      </c>
+      <c r="H80" s="2" t="inlineStr">
+        <is>
+          <t>مراجعة فقط</t>
+        </is>
+      </c>
+      <c r="I80" s="3" t="n">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="B81" s="2" t="inlineStr">
+        <is>
+          <t>الثلاثاء</t>
+        </is>
+      </c>
+      <c r="C81" s="2" t="inlineStr">
+        <is>
+          <t>السليل</t>
+        </is>
+      </c>
+      <c r="D81" s="2" t="n">
+        <v>35</v>
+      </c>
+      <c r="E81" s="2" t="inlineStr">
+        <is>
+          <t>د. الحسن الغنيمي</t>
+        </is>
+      </c>
+      <c r="F81" s="2" t="inlineStr"/>
+      <c r="G81" s="2" t="inlineStr">
+        <is>
+          <t>نعم</t>
+        </is>
+      </c>
+      <c r="H81" s="2" t="inlineStr">
+        <is>
+          <t>مراجعة فقط</t>
+        </is>
+      </c>
+      <c r="I81" s="3" t="n">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="B82" s="2" t="inlineStr">
+        <is>
+          <t>الثلاثاء</t>
+        </is>
+      </c>
+      <c r="C82" s="2" t="inlineStr">
+        <is>
+          <t>السليل</t>
+        </is>
+      </c>
+      <c r="D82" s="2" t="n">
+        <v>35</v>
+      </c>
+      <c r="E82" s="2" t="inlineStr">
+        <is>
+          <t>د. محمد جمال</t>
+        </is>
+      </c>
+      <c r="F82" s="2" t="inlineStr"/>
+      <c r="G82" s="2" t="inlineStr">
+        <is>
+          <t>نعم</t>
+        </is>
+      </c>
+      <c r="H82" s="2" t="inlineStr">
+        <is>
+          <t>مراجعة فقط</t>
+        </is>
+      </c>
+      <c r="I82" s="3" t="n">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="B83" s="2" t="inlineStr">
+        <is>
+          <t>الثلاثاء</t>
+        </is>
+      </c>
+      <c r="C83" s="2" t="inlineStr">
+        <is>
+          <t>السليل</t>
+        </is>
+      </c>
+      <c r="D83" s="2" t="n">
+        <v>53</v>
+      </c>
+      <c r="E83" s="2" t="inlineStr">
+        <is>
+          <t>د. حسام شلش</t>
+        </is>
+      </c>
+      <c r="F83" s="2" t="inlineStr">
+        <is>
+          <t>نعم</t>
+        </is>
+      </c>
+      <c r="G83" s="2" t="inlineStr">
+        <is>
+          <t>نعم</t>
+        </is>
+      </c>
+      <c r="H83" s="2" t="inlineStr">
+        <is>
+          <t>جرد + مراجعة</t>
+        </is>
+      </c>
+      <c r="I83" s="3" t="n">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="B84" s="2" t="inlineStr">
+        <is>
+          <t>الثلاثاء</t>
+        </is>
+      </c>
+      <c r="C84" s="2" t="inlineStr">
+        <is>
+          <t>السليل</t>
+        </is>
+      </c>
+      <c r="D84" s="2" t="n">
+        <v>53</v>
+      </c>
+      <c r="E84" s="2" t="inlineStr">
+        <is>
+          <t>د. السيد حسن</t>
+        </is>
+      </c>
+      <c r="F84" s="2" t="inlineStr"/>
+      <c r="G84" s="2" t="inlineStr">
+        <is>
+          <t>نعم</t>
+        </is>
+      </c>
+      <c r="H84" s="2" t="inlineStr">
+        <is>
+          <t>مراجعة فقط</t>
+        </is>
+      </c>
+      <c r="I84" s="3" t="n">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="B85" s="2" t="inlineStr">
+        <is>
+          <t>الثلاثاء</t>
+        </is>
+      </c>
+      <c r="C85" s="2" t="inlineStr">
+        <is>
+          <t>السليل</t>
+        </is>
+      </c>
+      <c r="D85" s="2" t="n">
+        <v>53</v>
+      </c>
+      <c r="E85" s="2" t="inlineStr">
+        <is>
+          <t>د. الحسن الغنيمي</t>
+        </is>
+      </c>
+      <c r="F85" s="2" t="inlineStr"/>
+      <c r="G85" s="2" t="inlineStr">
+        <is>
+          <t>نعم</t>
+        </is>
+      </c>
+      <c r="H85" s="2" t="inlineStr">
+        <is>
+          <t>مراجعة فقط</t>
+        </is>
+      </c>
+      <c r="I85" s="3" t="n">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="B86" s="2" t="inlineStr">
+        <is>
+          <t>الثلاثاء</t>
+        </is>
+      </c>
+      <c r="C86" s="2" t="inlineStr">
+        <is>
+          <t>السليل</t>
+        </is>
+      </c>
+      <c r="D86" s="2" t="n">
+        <v>53</v>
+      </c>
+      <c r="E86" s="2" t="inlineStr">
+        <is>
+          <t>د. محمد جمال</t>
+        </is>
+      </c>
+      <c r="F86" s="2" t="inlineStr"/>
+      <c r="G86" s="2" t="inlineStr">
+        <is>
+          <t>نعم</t>
+        </is>
+      </c>
+      <c r="H86" s="2" t="inlineStr">
+        <is>
+          <t>مراجعة فقط</t>
+        </is>
+      </c>
+      <c r="I86" s="3" t="n">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="4" t="inlineStr">
         <is>
           <t>الإجمالي</t>
         </is>
       </c>
-      <c r="B79" s="4" t="n"/>
-      <c r="C79" s="4" t="n"/>
-      <c r="D79" s="4" t="n"/>
-      <c r="E79" s="4" t="n"/>
-      <c r="F79" s="4" t="n"/>
-      <c r="G79" s="4" t="n"/>
-      <c r="H79" s="4" t="n"/>
-      <c r="I79" s="5">
-        <f>SUM(I2:I78)</f>
-        <v>12500</v>
+      <c r="B87" s="4" t="n"/>
+      <c r="C87" s="4" t="n"/>
+      <c r="D87" s="4" t="n"/>
+      <c r="E87" s="4" t="n"/>
+      <c r="F87" s="4" t="n"/>
+      <c r="G87" s="4" t="n"/>
+      <c r="H87" s="4" t="n"/>
+      <c r="I87" s="5">
+        <f>SUM(I2:I86)</f>
+        <v>13800</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:I78"/>
+  <autoFilter ref="A1:I86"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Log Oct 7 counts and reviews (pharmacies 46 and 56)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01RnF4y3zxCG7NcjFkMnYdwu
</commit_message>
<xml_diff>
--- a/inventory/jard_log.xlsx
+++ b/inventory/jard_log.xlsx
@@ -10,7 +10,7 @@
     <sheet name="السجل" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'السجل'!$A$1:$I$86</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'السجل'!$A$1:$I$94</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -468,7 +468,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I87"/>
+  <dimension ref="A1:I95"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -3929,25 +3929,345 @@
       </c>
     </row>
     <row r="87">
-      <c r="A87" s="4" t="inlineStr">
+      <c r="A87" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="B87" s="2" t="inlineStr">
+        <is>
+          <t>الأربعاء</t>
+        </is>
+      </c>
+      <c r="C87" s="2" t="inlineStr">
+        <is>
+          <t>تمرة - الدواسر</t>
+        </is>
+      </c>
+      <c r="D87" s="2" t="n">
+        <v>46</v>
+      </c>
+      <c r="E87" s="2" t="inlineStr">
+        <is>
+          <t>د. السيد حسن</t>
+        </is>
+      </c>
+      <c r="F87" s="2" t="inlineStr">
+        <is>
+          <t>نعم</t>
+        </is>
+      </c>
+      <c r="G87" s="2" t="inlineStr">
+        <is>
+          <t>نعم</t>
+        </is>
+      </c>
+      <c r="H87" s="2" t="inlineStr">
+        <is>
+          <t>جرد + مراجعة</t>
+        </is>
+      </c>
+      <c r="I87" s="3" t="n">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="B88" s="2" t="inlineStr">
+        <is>
+          <t>الأربعاء</t>
+        </is>
+      </c>
+      <c r="C88" s="2" t="inlineStr">
+        <is>
+          <t>تمرة - الدواسر</t>
+        </is>
+      </c>
+      <c r="D88" s="2" t="n">
+        <v>46</v>
+      </c>
+      <c r="E88" s="2" t="inlineStr">
+        <is>
+          <t>د. حسام شلش</t>
+        </is>
+      </c>
+      <c r="F88" s="2" t="inlineStr"/>
+      <c r="G88" s="2" t="inlineStr">
+        <is>
+          <t>نعم</t>
+        </is>
+      </c>
+      <c r="H88" s="2" t="inlineStr">
+        <is>
+          <t>مراجعة فقط</t>
+        </is>
+      </c>
+      <c r="I88" s="3" t="n">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="B89" s="2" t="inlineStr">
+        <is>
+          <t>الأربعاء</t>
+        </is>
+      </c>
+      <c r="C89" s="2" t="inlineStr">
+        <is>
+          <t>تمرة - الدواسر</t>
+        </is>
+      </c>
+      <c r="D89" s="2" t="n">
+        <v>46</v>
+      </c>
+      <c r="E89" s="2" t="inlineStr">
+        <is>
+          <t>د. الحسن الغنيمي</t>
+        </is>
+      </c>
+      <c r="F89" s="2" t="inlineStr"/>
+      <c r="G89" s="2" t="inlineStr">
+        <is>
+          <t>نعم</t>
+        </is>
+      </c>
+      <c r="H89" s="2" t="inlineStr">
+        <is>
+          <t>مراجعة فقط</t>
+        </is>
+      </c>
+      <c r="I89" s="3" t="n">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="B90" s="2" t="inlineStr">
+        <is>
+          <t>الأربعاء</t>
+        </is>
+      </c>
+      <c r="C90" s="2" t="inlineStr">
+        <is>
+          <t>تمرة - الدواسر</t>
+        </is>
+      </c>
+      <c r="D90" s="2" t="n">
+        <v>46</v>
+      </c>
+      <c r="E90" s="2" t="inlineStr">
+        <is>
+          <t>د. محمد جمال</t>
+        </is>
+      </c>
+      <c r="F90" s="2" t="inlineStr"/>
+      <c r="G90" s="2" t="inlineStr">
+        <is>
+          <t>نعم</t>
+        </is>
+      </c>
+      <c r="H90" s="2" t="inlineStr">
+        <is>
+          <t>مراجعة فقط</t>
+        </is>
+      </c>
+      <c r="I90" s="3" t="n">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="B91" s="2" t="inlineStr">
+        <is>
+          <t>الأربعاء</t>
+        </is>
+      </c>
+      <c r="C91" s="2" t="inlineStr">
+        <is>
+          <t>تمرة - الدواسر</t>
+        </is>
+      </c>
+      <c r="D91" s="2" t="n">
+        <v>56</v>
+      </c>
+      <c r="E91" s="2" t="inlineStr">
+        <is>
+          <t>د. السيد حسن</t>
+        </is>
+      </c>
+      <c r="F91" s="2" t="inlineStr">
+        <is>
+          <t>نعم</t>
+        </is>
+      </c>
+      <c r="G91" s="2" t="inlineStr">
+        <is>
+          <t>نعم</t>
+        </is>
+      </c>
+      <c r="H91" s="2" t="inlineStr">
+        <is>
+          <t>جرد + مراجعة</t>
+        </is>
+      </c>
+      <c r="I91" s="3" t="n">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="B92" s="2" t="inlineStr">
+        <is>
+          <t>الأربعاء</t>
+        </is>
+      </c>
+      <c r="C92" s="2" t="inlineStr">
+        <is>
+          <t>تمرة - الدواسر</t>
+        </is>
+      </c>
+      <c r="D92" s="2" t="n">
+        <v>56</v>
+      </c>
+      <c r="E92" s="2" t="inlineStr">
+        <is>
+          <t>د. حسام شلش</t>
+        </is>
+      </c>
+      <c r="F92" s="2" t="inlineStr"/>
+      <c r="G92" s="2" t="inlineStr">
+        <is>
+          <t>نعم</t>
+        </is>
+      </c>
+      <c r="H92" s="2" t="inlineStr">
+        <is>
+          <t>مراجعة فقط</t>
+        </is>
+      </c>
+      <c r="I92" s="3" t="n">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="B93" s="2" t="inlineStr">
+        <is>
+          <t>الأربعاء</t>
+        </is>
+      </c>
+      <c r="C93" s="2" t="inlineStr">
+        <is>
+          <t>تمرة - الدواسر</t>
+        </is>
+      </c>
+      <c r="D93" s="2" t="n">
+        <v>56</v>
+      </c>
+      <c r="E93" s="2" t="inlineStr">
+        <is>
+          <t>د. الحسن الغنيمي</t>
+        </is>
+      </c>
+      <c r="F93" s="2" t="inlineStr"/>
+      <c r="G93" s="2" t="inlineStr">
+        <is>
+          <t>نعم</t>
+        </is>
+      </c>
+      <c r="H93" s="2" t="inlineStr">
+        <is>
+          <t>مراجعة فقط</t>
+        </is>
+      </c>
+      <c r="I93" s="3" t="n">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="B94" s="2" t="inlineStr">
+        <is>
+          <t>الأربعاء</t>
+        </is>
+      </c>
+      <c r="C94" s="2" t="inlineStr">
+        <is>
+          <t>تمرة - الدواسر</t>
+        </is>
+      </c>
+      <c r="D94" s="2" t="n">
+        <v>56</v>
+      </c>
+      <c r="E94" s="2" t="inlineStr">
+        <is>
+          <t>د. محمد جمال</t>
+        </is>
+      </c>
+      <c r="F94" s="2" t="inlineStr"/>
+      <c r="G94" s="2" t="inlineStr">
+        <is>
+          <t>نعم</t>
+        </is>
+      </c>
+      <c r="H94" s="2" t="inlineStr">
+        <is>
+          <t>مراجعة فقط</t>
+        </is>
+      </c>
+      <c r="I94" s="3" t="n">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" s="4" t="inlineStr">
         <is>
           <t>الإجمالي</t>
         </is>
       </c>
-      <c r="B87" s="4" t="n"/>
-      <c r="C87" s="4" t="n"/>
-      <c r="D87" s="4" t="n"/>
-      <c r="E87" s="4" t="n"/>
-      <c r="F87" s="4" t="n"/>
-      <c r="G87" s="4" t="n"/>
-      <c r="H87" s="4" t="n"/>
-      <c r="I87" s="5">
-        <f>SUM(I2:I86)</f>
-        <v>13800</v>
+      <c r="B95" s="4" t="n"/>
+      <c r="C95" s="4" t="n"/>
+      <c r="D95" s="4" t="n"/>
+      <c r="E95" s="4" t="n"/>
+      <c r="F95" s="4" t="n"/>
+      <c r="G95" s="4" t="n"/>
+      <c r="H95" s="4" t="n"/>
+      <c r="I95" s="5">
+        <f>SUM(I2:I94)</f>
+        <v>15100</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:I86"/>
+  <autoFilter ref="A1:I94"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Log Oct 8 counts and reviews (pharmacies 47 and 37)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01RnF4y3zxCG7NcjFkMnYdwu
</commit_message>
<xml_diff>
--- a/inventory/jard_log.xlsx
+++ b/inventory/jard_log.xlsx
@@ -10,7 +10,7 @@
     <sheet name="السجل" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'السجل'!$A$1:$I$94</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'السجل'!$A$1:$I$102</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -468,7 +468,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I95"/>
+  <dimension ref="A1:I103"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -4249,25 +4249,345 @@
       </c>
     </row>
     <row r="95">
-      <c r="A95" s="4" t="inlineStr">
+      <c r="A95" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="B95" s="2" t="inlineStr">
+        <is>
+          <t>الخميس</t>
+        </is>
+      </c>
+      <c r="C95" s="2" t="inlineStr">
+        <is>
+          <t>الدواسر</t>
+        </is>
+      </c>
+      <c r="D95" s="2" t="n">
+        <v>47</v>
+      </c>
+      <c r="E95" s="2" t="inlineStr">
+        <is>
+          <t>د. حسام شلش</t>
+        </is>
+      </c>
+      <c r="F95" s="2" t="inlineStr">
+        <is>
+          <t>نعم</t>
+        </is>
+      </c>
+      <c r="G95" s="2" t="inlineStr">
+        <is>
+          <t>نعم</t>
+        </is>
+      </c>
+      <c r="H95" s="2" t="inlineStr">
+        <is>
+          <t>جرد + مراجعة</t>
+        </is>
+      </c>
+      <c r="I95" s="3" t="n">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="B96" s="2" t="inlineStr">
+        <is>
+          <t>الخميس</t>
+        </is>
+      </c>
+      <c r="C96" s="2" t="inlineStr">
+        <is>
+          <t>الدواسر</t>
+        </is>
+      </c>
+      <c r="D96" s="2" t="n">
+        <v>47</v>
+      </c>
+      <c r="E96" s="2" t="inlineStr">
+        <is>
+          <t>د. السيد حسن</t>
+        </is>
+      </c>
+      <c r="F96" s="2" t="inlineStr"/>
+      <c r="G96" s="2" t="inlineStr">
+        <is>
+          <t>نعم</t>
+        </is>
+      </c>
+      <c r="H96" s="2" t="inlineStr">
+        <is>
+          <t>مراجعة فقط</t>
+        </is>
+      </c>
+      <c r="I96" s="3" t="n">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="B97" s="2" t="inlineStr">
+        <is>
+          <t>الخميس</t>
+        </is>
+      </c>
+      <c r="C97" s="2" t="inlineStr">
+        <is>
+          <t>الدواسر</t>
+        </is>
+      </c>
+      <c r="D97" s="2" t="n">
+        <v>47</v>
+      </c>
+      <c r="E97" s="2" t="inlineStr">
+        <is>
+          <t>د. الحسن الغنيمي</t>
+        </is>
+      </c>
+      <c r="F97" s="2" t="inlineStr"/>
+      <c r="G97" s="2" t="inlineStr">
+        <is>
+          <t>نعم</t>
+        </is>
+      </c>
+      <c r="H97" s="2" t="inlineStr">
+        <is>
+          <t>مراجعة فقط</t>
+        </is>
+      </c>
+      <c r="I97" s="3" t="n">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="B98" s="2" t="inlineStr">
+        <is>
+          <t>الخميس</t>
+        </is>
+      </c>
+      <c r="C98" s="2" t="inlineStr">
+        <is>
+          <t>الدواسر</t>
+        </is>
+      </c>
+      <c r="D98" s="2" t="n">
+        <v>47</v>
+      </c>
+      <c r="E98" s="2" t="inlineStr">
+        <is>
+          <t>د. محمد جمال</t>
+        </is>
+      </c>
+      <c r="F98" s="2" t="inlineStr"/>
+      <c r="G98" s="2" t="inlineStr">
+        <is>
+          <t>نعم</t>
+        </is>
+      </c>
+      <c r="H98" s="2" t="inlineStr">
+        <is>
+          <t>مراجعة فقط</t>
+        </is>
+      </c>
+      <c r="I98" s="3" t="n">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="B99" s="2" t="inlineStr">
+        <is>
+          <t>الخميس</t>
+        </is>
+      </c>
+      <c r="C99" s="2" t="inlineStr">
+        <is>
+          <t>الدواسر</t>
+        </is>
+      </c>
+      <c r="D99" s="2" t="n">
+        <v>37</v>
+      </c>
+      <c r="E99" s="2" t="inlineStr">
+        <is>
+          <t>د. حسام شلش</t>
+        </is>
+      </c>
+      <c r="F99" s="2" t="inlineStr">
+        <is>
+          <t>نعم</t>
+        </is>
+      </c>
+      <c r="G99" s="2" t="inlineStr">
+        <is>
+          <t>نعم</t>
+        </is>
+      </c>
+      <c r="H99" s="2" t="inlineStr">
+        <is>
+          <t>جرد + مراجعة</t>
+        </is>
+      </c>
+      <c r="I99" s="3" t="n">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="B100" s="2" t="inlineStr">
+        <is>
+          <t>الخميس</t>
+        </is>
+      </c>
+      <c r="C100" s="2" t="inlineStr">
+        <is>
+          <t>الدواسر</t>
+        </is>
+      </c>
+      <c r="D100" s="2" t="n">
+        <v>37</v>
+      </c>
+      <c r="E100" s="2" t="inlineStr">
+        <is>
+          <t>د. السيد حسن</t>
+        </is>
+      </c>
+      <c r="F100" s="2" t="inlineStr"/>
+      <c r="G100" s="2" t="inlineStr">
+        <is>
+          <t>نعم</t>
+        </is>
+      </c>
+      <c r="H100" s="2" t="inlineStr">
+        <is>
+          <t>مراجعة فقط</t>
+        </is>
+      </c>
+      <c r="I100" s="3" t="n">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="B101" s="2" t="inlineStr">
+        <is>
+          <t>الخميس</t>
+        </is>
+      </c>
+      <c r="C101" s="2" t="inlineStr">
+        <is>
+          <t>الدواسر</t>
+        </is>
+      </c>
+      <c r="D101" s="2" t="n">
+        <v>37</v>
+      </c>
+      <c r="E101" s="2" t="inlineStr">
+        <is>
+          <t>د. الحسن الغنيمي</t>
+        </is>
+      </c>
+      <c r="F101" s="2" t="inlineStr"/>
+      <c r="G101" s="2" t="inlineStr">
+        <is>
+          <t>نعم</t>
+        </is>
+      </c>
+      <c r="H101" s="2" t="inlineStr">
+        <is>
+          <t>مراجعة فقط</t>
+        </is>
+      </c>
+      <c r="I101" s="3" t="n">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="B102" s="2" t="inlineStr">
+        <is>
+          <t>الخميس</t>
+        </is>
+      </c>
+      <c r="C102" s="2" t="inlineStr">
+        <is>
+          <t>الدواسر</t>
+        </is>
+      </c>
+      <c r="D102" s="2" t="n">
+        <v>37</v>
+      </c>
+      <c r="E102" s="2" t="inlineStr">
+        <is>
+          <t>د. محمد جمال</t>
+        </is>
+      </c>
+      <c r="F102" s="2" t="inlineStr"/>
+      <c r="G102" s="2" t="inlineStr">
+        <is>
+          <t>نعم</t>
+        </is>
+      </c>
+      <c r="H102" s="2" t="inlineStr">
+        <is>
+          <t>مراجعة فقط</t>
+        </is>
+      </c>
+      <c r="I102" s="3" t="n">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" s="4" t="inlineStr">
         <is>
           <t>الإجمالي</t>
         </is>
       </c>
-      <c r="B95" s="4" t="n"/>
-      <c r="C95" s="4" t="n"/>
-      <c r="D95" s="4" t="n"/>
-      <c r="E95" s="4" t="n"/>
-      <c r="F95" s="4" t="n"/>
-      <c r="G95" s="4" t="n"/>
-      <c r="H95" s="4" t="n"/>
-      <c r="I95" s="5">
-        <f>SUM(I2:I94)</f>
-        <v>15100</v>
+      <c r="B103" s="4" t="n"/>
+      <c r="C103" s="4" t="n"/>
+      <c r="D103" s="4" t="n"/>
+      <c r="E103" s="4" t="n"/>
+      <c r="F103" s="4" t="n"/>
+      <c r="G103" s="4" t="n"/>
+      <c r="H103" s="4" t="n"/>
+      <c r="I103" s="5">
+        <f>SUM(I2:I102)</f>
+        <v>16400</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:I94"/>
+  <autoFilter ref="A1:I102"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Log Oct 9 counts and reviews (pharmacies 38 and 59)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01RnF4y3zxCG7NcjFkMnYdwu
</commit_message>
<xml_diff>
--- a/inventory/jard_log.xlsx
+++ b/inventory/jard_log.xlsx
@@ -10,7 +10,7 @@
     <sheet name="السجل" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'السجل'!$A$1:$I$102</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'السجل'!$A$1:$I$110</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -468,7 +468,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I103"/>
+  <dimension ref="A1:I111"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -4569,25 +4569,345 @@
       </c>
     </row>
     <row r="103">
-      <c r="A103" s="4" t="inlineStr">
+      <c r="A103" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="B103" s="2" t="inlineStr">
+        <is>
+          <t>الجمعة</t>
+        </is>
+      </c>
+      <c r="C103" s="2" t="inlineStr">
+        <is>
+          <t>الدواسر</t>
+        </is>
+      </c>
+      <c r="D103" s="2" t="n">
+        <v>38</v>
+      </c>
+      <c r="E103" s="2" t="inlineStr">
+        <is>
+          <t>د. السيد حسن</t>
+        </is>
+      </c>
+      <c r="F103" s="2" t="inlineStr">
+        <is>
+          <t>نعم</t>
+        </is>
+      </c>
+      <c r="G103" s="2" t="inlineStr">
+        <is>
+          <t>نعم</t>
+        </is>
+      </c>
+      <c r="H103" s="2" t="inlineStr">
+        <is>
+          <t>جرد + مراجعة</t>
+        </is>
+      </c>
+      <c r="I103" s="3" t="n">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="B104" s="2" t="inlineStr">
+        <is>
+          <t>الجمعة</t>
+        </is>
+      </c>
+      <c r="C104" s="2" t="inlineStr">
+        <is>
+          <t>الدواسر</t>
+        </is>
+      </c>
+      <c r="D104" s="2" t="n">
+        <v>38</v>
+      </c>
+      <c r="E104" s="2" t="inlineStr">
+        <is>
+          <t>د. حسام شلش</t>
+        </is>
+      </c>
+      <c r="F104" s="2" t="inlineStr"/>
+      <c r="G104" s="2" t="inlineStr">
+        <is>
+          <t>نعم</t>
+        </is>
+      </c>
+      <c r="H104" s="2" t="inlineStr">
+        <is>
+          <t>مراجعة فقط</t>
+        </is>
+      </c>
+      <c r="I104" s="3" t="n">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="B105" s="2" t="inlineStr">
+        <is>
+          <t>الجمعة</t>
+        </is>
+      </c>
+      <c r="C105" s="2" t="inlineStr">
+        <is>
+          <t>الدواسر</t>
+        </is>
+      </c>
+      <c r="D105" s="2" t="n">
+        <v>38</v>
+      </c>
+      <c r="E105" s="2" t="inlineStr">
+        <is>
+          <t>د. الحسن الغنيمي</t>
+        </is>
+      </c>
+      <c r="F105" s="2" t="inlineStr"/>
+      <c r="G105" s="2" t="inlineStr">
+        <is>
+          <t>نعم</t>
+        </is>
+      </c>
+      <c r="H105" s="2" t="inlineStr">
+        <is>
+          <t>مراجعة فقط</t>
+        </is>
+      </c>
+      <c r="I105" s="3" t="n">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="B106" s="2" t="inlineStr">
+        <is>
+          <t>الجمعة</t>
+        </is>
+      </c>
+      <c r="C106" s="2" t="inlineStr">
+        <is>
+          <t>الدواسر</t>
+        </is>
+      </c>
+      <c r="D106" s="2" t="n">
+        <v>38</v>
+      </c>
+      <c r="E106" s="2" t="inlineStr">
+        <is>
+          <t>د. محمد جمال</t>
+        </is>
+      </c>
+      <c r="F106" s="2" t="inlineStr"/>
+      <c r="G106" s="2" t="inlineStr">
+        <is>
+          <t>نعم</t>
+        </is>
+      </c>
+      <c r="H106" s="2" t="inlineStr">
+        <is>
+          <t>مراجعة فقط</t>
+        </is>
+      </c>
+      <c r="I106" s="3" t="n">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="B107" s="2" t="inlineStr">
+        <is>
+          <t>الجمعة</t>
+        </is>
+      </c>
+      <c r="C107" s="2" t="inlineStr">
+        <is>
+          <t>الدواسر</t>
+        </is>
+      </c>
+      <c r="D107" s="2" t="n">
+        <v>59</v>
+      </c>
+      <c r="E107" s="2" t="inlineStr">
+        <is>
+          <t>د. السيد حسن</t>
+        </is>
+      </c>
+      <c r="F107" s="2" t="inlineStr">
+        <is>
+          <t>نعم</t>
+        </is>
+      </c>
+      <c r="G107" s="2" t="inlineStr">
+        <is>
+          <t>نعم</t>
+        </is>
+      </c>
+      <c r="H107" s="2" t="inlineStr">
+        <is>
+          <t>جرد + مراجعة</t>
+        </is>
+      </c>
+      <c r="I107" s="3" t="n">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="B108" s="2" t="inlineStr">
+        <is>
+          <t>الجمعة</t>
+        </is>
+      </c>
+      <c r="C108" s="2" t="inlineStr">
+        <is>
+          <t>الدواسر</t>
+        </is>
+      </c>
+      <c r="D108" s="2" t="n">
+        <v>59</v>
+      </c>
+      <c r="E108" s="2" t="inlineStr">
+        <is>
+          <t>د. حسام شلش</t>
+        </is>
+      </c>
+      <c r="F108" s="2" t="inlineStr"/>
+      <c r="G108" s="2" t="inlineStr">
+        <is>
+          <t>نعم</t>
+        </is>
+      </c>
+      <c r="H108" s="2" t="inlineStr">
+        <is>
+          <t>مراجعة فقط</t>
+        </is>
+      </c>
+      <c r="I108" s="3" t="n">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="B109" s="2" t="inlineStr">
+        <is>
+          <t>الجمعة</t>
+        </is>
+      </c>
+      <c r="C109" s="2" t="inlineStr">
+        <is>
+          <t>الدواسر</t>
+        </is>
+      </c>
+      <c r="D109" s="2" t="n">
+        <v>59</v>
+      </c>
+      <c r="E109" s="2" t="inlineStr">
+        <is>
+          <t>د. الحسن الغنيمي</t>
+        </is>
+      </c>
+      <c r="F109" s="2" t="inlineStr"/>
+      <c r="G109" s="2" t="inlineStr">
+        <is>
+          <t>نعم</t>
+        </is>
+      </c>
+      <c r="H109" s="2" t="inlineStr">
+        <is>
+          <t>مراجعة فقط</t>
+        </is>
+      </c>
+      <c r="I109" s="3" t="n">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="B110" s="2" t="inlineStr">
+        <is>
+          <t>الجمعة</t>
+        </is>
+      </c>
+      <c r="C110" s="2" t="inlineStr">
+        <is>
+          <t>الدواسر</t>
+        </is>
+      </c>
+      <c r="D110" s="2" t="n">
+        <v>59</v>
+      </c>
+      <c r="E110" s="2" t="inlineStr">
+        <is>
+          <t>د. محمد جمال</t>
+        </is>
+      </c>
+      <c r="F110" s="2" t="inlineStr"/>
+      <c r="G110" s="2" t="inlineStr">
+        <is>
+          <t>نعم</t>
+        </is>
+      </c>
+      <c r="H110" s="2" t="inlineStr">
+        <is>
+          <t>مراجعة فقط</t>
+        </is>
+      </c>
+      <c r="I110" s="3" t="n">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" s="4" t="inlineStr">
         <is>
           <t>الإجمالي</t>
         </is>
       </c>
-      <c r="B103" s="4" t="n"/>
-      <c r="C103" s="4" t="n"/>
-      <c r="D103" s="4" t="n"/>
-      <c r="E103" s="4" t="n"/>
-      <c r="F103" s="4" t="n"/>
-      <c r="G103" s="4" t="n"/>
-      <c r="H103" s="4" t="n"/>
-      <c r="I103" s="5">
-        <f>SUM(I2:I102)</f>
-        <v>16400</v>
+      <c r="B111" s="4" t="n"/>
+      <c r="C111" s="4" t="n"/>
+      <c r="D111" s="4" t="n"/>
+      <c r="E111" s="4" t="n"/>
+      <c r="F111" s="4" t="n"/>
+      <c r="G111" s="4" t="n"/>
+      <c r="H111" s="4" t="n"/>
+      <c r="I111" s="5">
+        <f>SUM(I2:I110)</f>
+        <v>17700</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:I102"/>
+  <autoFilter ref="A1:I110"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Log Oct 10 counts and reviews (pharmacies 36 and 57)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01RnF4y3zxCG7NcjFkMnYdwu
</commit_message>
<xml_diff>
--- a/inventory/jard_log.xlsx
+++ b/inventory/jard_log.xlsx
@@ -10,7 +10,7 @@
     <sheet name="السجل" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'السجل'!$A$1:$I$110</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'السجل'!$A$1:$I$118</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -468,7 +468,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I111"/>
+  <dimension ref="A1:I119"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -4889,25 +4889,345 @@
       </c>
     </row>
     <row r="111">
-      <c r="A111" s="4" t="inlineStr">
+      <c r="A111" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="B111" s="2" t="inlineStr">
+        <is>
+          <t>السبت</t>
+        </is>
+      </c>
+      <c r="C111" s="2" t="inlineStr">
+        <is>
+          <t>الدواسر</t>
+        </is>
+      </c>
+      <c r="D111" s="2" t="n">
+        <v>36</v>
+      </c>
+      <c r="E111" s="2" t="inlineStr">
+        <is>
+          <t>د. حسام شلش</t>
+        </is>
+      </c>
+      <c r="F111" s="2" t="inlineStr">
+        <is>
+          <t>نعم</t>
+        </is>
+      </c>
+      <c r="G111" s="2" t="inlineStr">
+        <is>
+          <t>نعم</t>
+        </is>
+      </c>
+      <c r="H111" s="2" t="inlineStr">
+        <is>
+          <t>جرد + مراجعة</t>
+        </is>
+      </c>
+      <c r="I111" s="3" t="n">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="B112" s="2" t="inlineStr">
+        <is>
+          <t>السبت</t>
+        </is>
+      </c>
+      <c r="C112" s="2" t="inlineStr">
+        <is>
+          <t>الدواسر</t>
+        </is>
+      </c>
+      <c r="D112" s="2" t="n">
+        <v>36</v>
+      </c>
+      <c r="E112" s="2" t="inlineStr">
+        <is>
+          <t>د. السيد حسن</t>
+        </is>
+      </c>
+      <c r="F112" s="2" t="inlineStr"/>
+      <c r="G112" s="2" t="inlineStr">
+        <is>
+          <t>نعم</t>
+        </is>
+      </c>
+      <c r="H112" s="2" t="inlineStr">
+        <is>
+          <t>مراجعة فقط</t>
+        </is>
+      </c>
+      <c r="I112" s="3" t="n">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="B113" s="2" t="inlineStr">
+        <is>
+          <t>السبت</t>
+        </is>
+      </c>
+      <c r="C113" s="2" t="inlineStr">
+        <is>
+          <t>الدواسر</t>
+        </is>
+      </c>
+      <c r="D113" s="2" t="n">
+        <v>36</v>
+      </c>
+      <c r="E113" s="2" t="inlineStr">
+        <is>
+          <t>د. الحسن الغنيمي</t>
+        </is>
+      </c>
+      <c r="F113" s="2" t="inlineStr"/>
+      <c r="G113" s="2" t="inlineStr">
+        <is>
+          <t>نعم</t>
+        </is>
+      </c>
+      <c r="H113" s="2" t="inlineStr">
+        <is>
+          <t>مراجعة فقط</t>
+        </is>
+      </c>
+      <c r="I113" s="3" t="n">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="B114" s="2" t="inlineStr">
+        <is>
+          <t>السبت</t>
+        </is>
+      </c>
+      <c r="C114" s="2" t="inlineStr">
+        <is>
+          <t>الدواسر</t>
+        </is>
+      </c>
+      <c r="D114" s="2" t="n">
+        <v>36</v>
+      </c>
+      <c r="E114" s="2" t="inlineStr">
+        <is>
+          <t>د. محمد جمال</t>
+        </is>
+      </c>
+      <c r="F114" s="2" t="inlineStr"/>
+      <c r="G114" s="2" t="inlineStr">
+        <is>
+          <t>نعم</t>
+        </is>
+      </c>
+      <c r="H114" s="2" t="inlineStr">
+        <is>
+          <t>مراجعة فقط</t>
+        </is>
+      </c>
+      <c r="I114" s="3" t="n">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="B115" s="2" t="inlineStr">
+        <is>
+          <t>السبت</t>
+        </is>
+      </c>
+      <c r="C115" s="2" t="inlineStr">
+        <is>
+          <t>الدواسر</t>
+        </is>
+      </c>
+      <c r="D115" s="2" t="n">
+        <v>57</v>
+      </c>
+      <c r="E115" s="2" t="inlineStr">
+        <is>
+          <t>د. حسام شلش</t>
+        </is>
+      </c>
+      <c r="F115" s="2" t="inlineStr">
+        <is>
+          <t>نعم</t>
+        </is>
+      </c>
+      <c r="G115" s="2" t="inlineStr">
+        <is>
+          <t>نعم</t>
+        </is>
+      </c>
+      <c r="H115" s="2" t="inlineStr">
+        <is>
+          <t>جرد + مراجعة</t>
+        </is>
+      </c>
+      <c r="I115" s="3" t="n">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="B116" s="2" t="inlineStr">
+        <is>
+          <t>السبت</t>
+        </is>
+      </c>
+      <c r="C116" s="2" t="inlineStr">
+        <is>
+          <t>الدواسر</t>
+        </is>
+      </c>
+      <c r="D116" s="2" t="n">
+        <v>57</v>
+      </c>
+      <c r="E116" s="2" t="inlineStr">
+        <is>
+          <t>د. السيد حسن</t>
+        </is>
+      </c>
+      <c r="F116" s="2" t="inlineStr"/>
+      <c r="G116" s="2" t="inlineStr">
+        <is>
+          <t>نعم</t>
+        </is>
+      </c>
+      <c r="H116" s="2" t="inlineStr">
+        <is>
+          <t>مراجعة فقط</t>
+        </is>
+      </c>
+      <c r="I116" s="3" t="n">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="B117" s="2" t="inlineStr">
+        <is>
+          <t>السبت</t>
+        </is>
+      </c>
+      <c r="C117" s="2" t="inlineStr">
+        <is>
+          <t>الدواسر</t>
+        </is>
+      </c>
+      <c r="D117" s="2" t="n">
+        <v>57</v>
+      </c>
+      <c r="E117" s="2" t="inlineStr">
+        <is>
+          <t>د. الحسن الغنيمي</t>
+        </is>
+      </c>
+      <c r="F117" s="2" t="inlineStr"/>
+      <c r="G117" s="2" t="inlineStr">
+        <is>
+          <t>نعم</t>
+        </is>
+      </c>
+      <c r="H117" s="2" t="inlineStr">
+        <is>
+          <t>مراجعة فقط</t>
+        </is>
+      </c>
+      <c r="I117" s="3" t="n">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="B118" s="2" t="inlineStr">
+        <is>
+          <t>السبت</t>
+        </is>
+      </c>
+      <c r="C118" s="2" t="inlineStr">
+        <is>
+          <t>الدواسر</t>
+        </is>
+      </c>
+      <c r="D118" s="2" t="n">
+        <v>57</v>
+      </c>
+      <c r="E118" s="2" t="inlineStr">
+        <is>
+          <t>د. محمد جمال</t>
+        </is>
+      </c>
+      <c r="F118" s="2" t="inlineStr"/>
+      <c r="G118" s="2" t="inlineStr">
+        <is>
+          <t>نعم</t>
+        </is>
+      </c>
+      <c r="H118" s="2" t="inlineStr">
+        <is>
+          <t>مراجعة فقط</t>
+        </is>
+      </c>
+      <c r="I118" s="3" t="n">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" s="4" t="inlineStr">
         <is>
           <t>الإجمالي</t>
         </is>
       </c>
-      <c r="B111" s="4" t="n"/>
-      <c r="C111" s="4" t="n"/>
-      <c r="D111" s="4" t="n"/>
-      <c r="E111" s="4" t="n"/>
-      <c r="F111" s="4" t="n"/>
-      <c r="G111" s="4" t="n"/>
-      <c r="H111" s="4" t="n"/>
-      <c r="I111" s="5">
-        <f>SUM(I2:I110)</f>
-        <v>17700</v>
+      <c r="B119" s="4" t="n"/>
+      <c r="C119" s="4" t="n"/>
+      <c r="D119" s="4" t="n"/>
+      <c r="E119" s="4" t="n"/>
+      <c r="F119" s="4" t="n"/>
+      <c r="G119" s="4" t="n"/>
+      <c r="H119" s="4" t="n"/>
+      <c r="I119" s="5">
+        <f>SUM(I2:I118)</f>
+        <v>19000</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:I110"/>
+  <autoFilter ref="A1:I118"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Log Oct 11 counts and reviews in Ranyah (pharmacies 48 and 49)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01RnF4y3zxCG7NcjFkMnYdwu
</commit_message>
<xml_diff>
--- a/inventory/jard_log.xlsx
+++ b/inventory/jard_log.xlsx
@@ -10,7 +10,7 @@
     <sheet name="السجل" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'السجل'!$A$1:$I$118</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'السجل'!$A$1:$I$126</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -468,7 +468,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I119"/>
+  <dimension ref="A1:I127"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -5209,25 +5209,345 @@
       </c>
     </row>
     <row r="119">
-      <c r="A119" s="4" t="inlineStr">
+      <c r="A119" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-11</t>
+        </is>
+      </c>
+      <c r="B119" s="2" t="inlineStr">
+        <is>
+          <t>الأحد</t>
+        </is>
+      </c>
+      <c r="C119" s="2" t="inlineStr">
+        <is>
+          <t>رنية</t>
+        </is>
+      </c>
+      <c r="D119" s="2" t="n">
+        <v>48</v>
+      </c>
+      <c r="E119" s="2" t="inlineStr">
+        <is>
+          <t>د. السيد حسن</t>
+        </is>
+      </c>
+      <c r="F119" s="2" t="inlineStr">
+        <is>
+          <t>نعم</t>
+        </is>
+      </c>
+      <c r="G119" s="2" t="inlineStr">
+        <is>
+          <t>نعم</t>
+        </is>
+      </c>
+      <c r="H119" s="2" t="inlineStr">
+        <is>
+          <t>جرد + مراجعة</t>
+        </is>
+      </c>
+      <c r="I119" s="3" t="n">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-11</t>
+        </is>
+      </c>
+      <c r="B120" s="2" t="inlineStr">
+        <is>
+          <t>الأحد</t>
+        </is>
+      </c>
+      <c r="C120" s="2" t="inlineStr">
+        <is>
+          <t>رنية</t>
+        </is>
+      </c>
+      <c r="D120" s="2" t="n">
+        <v>48</v>
+      </c>
+      <c r="E120" s="2" t="inlineStr">
+        <is>
+          <t>د. حسام شلش</t>
+        </is>
+      </c>
+      <c r="F120" s="2" t="inlineStr"/>
+      <c r="G120" s="2" t="inlineStr">
+        <is>
+          <t>نعم</t>
+        </is>
+      </c>
+      <c r="H120" s="2" t="inlineStr">
+        <is>
+          <t>مراجعة فقط</t>
+        </is>
+      </c>
+      <c r="I120" s="3" t="n">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-11</t>
+        </is>
+      </c>
+      <c r="B121" s="2" t="inlineStr">
+        <is>
+          <t>الأحد</t>
+        </is>
+      </c>
+      <c r="C121" s="2" t="inlineStr">
+        <is>
+          <t>رنية</t>
+        </is>
+      </c>
+      <c r="D121" s="2" t="n">
+        <v>48</v>
+      </c>
+      <c r="E121" s="2" t="inlineStr">
+        <is>
+          <t>د. الحسن الغنيمي</t>
+        </is>
+      </c>
+      <c r="F121" s="2" t="inlineStr"/>
+      <c r="G121" s="2" t="inlineStr">
+        <is>
+          <t>نعم</t>
+        </is>
+      </c>
+      <c r="H121" s="2" t="inlineStr">
+        <is>
+          <t>مراجعة فقط</t>
+        </is>
+      </c>
+      <c r="I121" s="3" t="n">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-11</t>
+        </is>
+      </c>
+      <c r="B122" s="2" t="inlineStr">
+        <is>
+          <t>الأحد</t>
+        </is>
+      </c>
+      <c r="C122" s="2" t="inlineStr">
+        <is>
+          <t>رنية</t>
+        </is>
+      </c>
+      <c r="D122" s="2" t="n">
+        <v>48</v>
+      </c>
+      <c r="E122" s="2" t="inlineStr">
+        <is>
+          <t>د. محمد جمال</t>
+        </is>
+      </c>
+      <c r="F122" s="2" t="inlineStr"/>
+      <c r="G122" s="2" t="inlineStr">
+        <is>
+          <t>نعم</t>
+        </is>
+      </c>
+      <c r="H122" s="2" t="inlineStr">
+        <is>
+          <t>مراجعة فقط</t>
+        </is>
+      </c>
+      <c r="I122" s="3" t="n">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-11</t>
+        </is>
+      </c>
+      <c r="B123" s="2" t="inlineStr">
+        <is>
+          <t>الأحد</t>
+        </is>
+      </c>
+      <c r="C123" s="2" t="inlineStr">
+        <is>
+          <t>رنية</t>
+        </is>
+      </c>
+      <c r="D123" s="2" t="n">
+        <v>49</v>
+      </c>
+      <c r="E123" s="2" t="inlineStr">
+        <is>
+          <t>د. السيد حسن</t>
+        </is>
+      </c>
+      <c r="F123" s="2" t="inlineStr">
+        <is>
+          <t>نعم</t>
+        </is>
+      </c>
+      <c r="G123" s="2" t="inlineStr">
+        <is>
+          <t>نعم</t>
+        </is>
+      </c>
+      <c r="H123" s="2" t="inlineStr">
+        <is>
+          <t>جرد + مراجعة</t>
+        </is>
+      </c>
+      <c r="I123" s="3" t="n">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-11</t>
+        </is>
+      </c>
+      <c r="B124" s="2" t="inlineStr">
+        <is>
+          <t>الأحد</t>
+        </is>
+      </c>
+      <c r="C124" s="2" t="inlineStr">
+        <is>
+          <t>رنية</t>
+        </is>
+      </c>
+      <c r="D124" s="2" t="n">
+        <v>49</v>
+      </c>
+      <c r="E124" s="2" t="inlineStr">
+        <is>
+          <t>د. حسام شلش</t>
+        </is>
+      </c>
+      <c r="F124" s="2" t="inlineStr"/>
+      <c r="G124" s="2" t="inlineStr">
+        <is>
+          <t>نعم</t>
+        </is>
+      </c>
+      <c r="H124" s="2" t="inlineStr">
+        <is>
+          <t>مراجعة فقط</t>
+        </is>
+      </c>
+      <c r="I124" s="3" t="n">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-11</t>
+        </is>
+      </c>
+      <c r="B125" s="2" t="inlineStr">
+        <is>
+          <t>الأحد</t>
+        </is>
+      </c>
+      <c r="C125" s="2" t="inlineStr">
+        <is>
+          <t>رنية</t>
+        </is>
+      </c>
+      <c r="D125" s="2" t="n">
+        <v>49</v>
+      </c>
+      <c r="E125" s="2" t="inlineStr">
+        <is>
+          <t>د. الحسن الغنيمي</t>
+        </is>
+      </c>
+      <c r="F125" s="2" t="inlineStr"/>
+      <c r="G125" s="2" t="inlineStr">
+        <is>
+          <t>نعم</t>
+        </is>
+      </c>
+      <c r="H125" s="2" t="inlineStr">
+        <is>
+          <t>مراجعة فقط</t>
+        </is>
+      </c>
+      <c r="I125" s="3" t="n">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-11</t>
+        </is>
+      </c>
+      <c r="B126" s="2" t="inlineStr">
+        <is>
+          <t>الأحد</t>
+        </is>
+      </c>
+      <c r="C126" s="2" t="inlineStr">
+        <is>
+          <t>رنية</t>
+        </is>
+      </c>
+      <c r="D126" s="2" t="n">
+        <v>49</v>
+      </c>
+      <c r="E126" s="2" t="inlineStr">
+        <is>
+          <t>د. محمد جمال</t>
+        </is>
+      </c>
+      <c r="F126" s="2" t="inlineStr"/>
+      <c r="G126" s="2" t="inlineStr">
+        <is>
+          <t>نعم</t>
+        </is>
+      </c>
+      <c r="H126" s="2" t="inlineStr">
+        <is>
+          <t>مراجعة فقط</t>
+        </is>
+      </c>
+      <c r="I126" s="3" t="n">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" s="4" t="inlineStr">
         <is>
           <t>الإجمالي</t>
         </is>
       </c>
-      <c r="B119" s="4" t="n"/>
-      <c r="C119" s="4" t="n"/>
-      <c r="D119" s="4" t="n"/>
-      <c r="E119" s="4" t="n"/>
-      <c r="F119" s="4" t="n"/>
-      <c r="G119" s="4" t="n"/>
-      <c r="H119" s="4" t="n"/>
-      <c r="I119" s="5">
-        <f>SUM(I2:I118)</f>
-        <v>19000</v>
+      <c r="B127" s="4" t="n"/>
+      <c r="C127" s="4" t="n"/>
+      <c r="D127" s="4" t="n"/>
+      <c r="E127" s="4" t="n"/>
+      <c r="F127" s="4" t="n"/>
+      <c r="G127" s="4" t="n"/>
+      <c r="H127" s="4" t="n"/>
+      <c r="I127" s="5">
+        <f>SUM(I2:I126)</f>
+        <v>20300</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:I118"/>
+  <autoFilter ref="A1:I126"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Log Oct 13 counts and reviews (pharmacies 8 and 60)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01RnF4y3zxCG7NcjFkMnYdwu
</commit_message>
<xml_diff>
--- a/inventory/jard_log.xlsx
+++ b/inventory/jard_log.xlsx
@@ -10,7 +10,7 @@
     <sheet name="السجل" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'السجل'!$A$1:$I$126</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'السجل'!$A$1:$I$134</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -468,7 +468,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I127"/>
+  <dimension ref="A1:I135"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -5529,25 +5529,345 @@
       </c>
     </row>
     <row r="127">
-      <c r="A127" s="4" t="inlineStr">
+      <c r="A127" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="B127" s="2" t="inlineStr">
+        <is>
+          <t>الثلاثاء</t>
+        </is>
+      </c>
+      <c r="C127" s="2" t="inlineStr">
+        <is>
+          <t>الخرج</t>
+        </is>
+      </c>
+      <c r="D127" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="E127" s="2" t="inlineStr">
+        <is>
+          <t>د. علي خليفة</t>
+        </is>
+      </c>
+      <c r="F127" s="2" t="inlineStr">
+        <is>
+          <t>نعم</t>
+        </is>
+      </c>
+      <c r="G127" s="2" t="inlineStr">
+        <is>
+          <t>نعم</t>
+        </is>
+      </c>
+      <c r="H127" s="2" t="inlineStr">
+        <is>
+          <t>جرد + مراجعة</t>
+        </is>
+      </c>
+      <c r="I127" s="3" t="n">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="B128" s="2" t="inlineStr">
+        <is>
+          <t>الثلاثاء</t>
+        </is>
+      </c>
+      <c r="C128" s="2" t="inlineStr">
+        <is>
+          <t>الخرج</t>
+        </is>
+      </c>
+      <c r="D128" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="E128" s="2" t="inlineStr">
+        <is>
+          <t>د. السيد حسن</t>
+        </is>
+      </c>
+      <c r="F128" s="2" t="inlineStr"/>
+      <c r="G128" s="2" t="inlineStr">
+        <is>
+          <t>نعم</t>
+        </is>
+      </c>
+      <c r="H128" s="2" t="inlineStr">
+        <is>
+          <t>مراجعة فقط</t>
+        </is>
+      </c>
+      <c r="I128" s="3" t="n">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="B129" s="2" t="inlineStr">
+        <is>
+          <t>الثلاثاء</t>
+        </is>
+      </c>
+      <c r="C129" s="2" t="inlineStr">
+        <is>
+          <t>الخرج</t>
+        </is>
+      </c>
+      <c r="D129" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="E129" s="2" t="inlineStr">
+        <is>
+          <t>د. محمد جمال</t>
+        </is>
+      </c>
+      <c r="F129" s="2" t="inlineStr"/>
+      <c r="G129" s="2" t="inlineStr">
+        <is>
+          <t>نعم</t>
+        </is>
+      </c>
+      <c r="H129" s="2" t="inlineStr">
+        <is>
+          <t>مراجعة فقط</t>
+        </is>
+      </c>
+      <c r="I129" s="3" t="n">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="B130" s="2" t="inlineStr">
+        <is>
+          <t>الثلاثاء</t>
+        </is>
+      </c>
+      <c r="C130" s="2" t="inlineStr">
+        <is>
+          <t>الخرج</t>
+        </is>
+      </c>
+      <c r="D130" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="E130" s="2" t="inlineStr">
+        <is>
+          <t>د. حسام شلش</t>
+        </is>
+      </c>
+      <c r="F130" s="2" t="inlineStr"/>
+      <c r="G130" s="2" t="inlineStr">
+        <is>
+          <t>نعم</t>
+        </is>
+      </c>
+      <c r="H130" s="2" t="inlineStr">
+        <is>
+          <t>مراجعة فقط</t>
+        </is>
+      </c>
+      <c r="I130" s="3" t="n">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="B131" s="2" t="inlineStr">
+        <is>
+          <t>الثلاثاء</t>
+        </is>
+      </c>
+      <c r="C131" s="2" t="inlineStr">
+        <is>
+          <t>الخرج</t>
+        </is>
+      </c>
+      <c r="D131" s="2" t="n">
+        <v>60</v>
+      </c>
+      <c r="E131" s="2" t="inlineStr">
+        <is>
+          <t>د. علي خليفة</t>
+        </is>
+      </c>
+      <c r="F131" s="2" t="inlineStr">
+        <is>
+          <t>نعم</t>
+        </is>
+      </c>
+      <c r="G131" s="2" t="inlineStr">
+        <is>
+          <t>نعم</t>
+        </is>
+      </c>
+      <c r="H131" s="2" t="inlineStr">
+        <is>
+          <t>جرد + مراجعة</t>
+        </is>
+      </c>
+      <c r="I131" s="3" t="n">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="B132" s="2" t="inlineStr">
+        <is>
+          <t>الثلاثاء</t>
+        </is>
+      </c>
+      <c r="C132" s="2" t="inlineStr">
+        <is>
+          <t>الخرج</t>
+        </is>
+      </c>
+      <c r="D132" s="2" t="n">
+        <v>60</v>
+      </c>
+      <c r="E132" s="2" t="inlineStr">
+        <is>
+          <t>د. السيد حسن</t>
+        </is>
+      </c>
+      <c r="F132" s="2" t="inlineStr"/>
+      <c r="G132" s="2" t="inlineStr">
+        <is>
+          <t>نعم</t>
+        </is>
+      </c>
+      <c r="H132" s="2" t="inlineStr">
+        <is>
+          <t>مراجعة فقط</t>
+        </is>
+      </c>
+      <c r="I132" s="3" t="n">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="B133" s="2" t="inlineStr">
+        <is>
+          <t>الثلاثاء</t>
+        </is>
+      </c>
+      <c r="C133" s="2" t="inlineStr">
+        <is>
+          <t>الخرج</t>
+        </is>
+      </c>
+      <c r="D133" s="2" t="n">
+        <v>60</v>
+      </c>
+      <c r="E133" s="2" t="inlineStr">
+        <is>
+          <t>د. محمد جمال</t>
+        </is>
+      </c>
+      <c r="F133" s="2" t="inlineStr"/>
+      <c r="G133" s="2" t="inlineStr">
+        <is>
+          <t>نعم</t>
+        </is>
+      </c>
+      <c r="H133" s="2" t="inlineStr">
+        <is>
+          <t>مراجعة فقط</t>
+        </is>
+      </c>
+      <c r="I133" s="3" t="n">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="B134" s="2" t="inlineStr">
+        <is>
+          <t>الثلاثاء</t>
+        </is>
+      </c>
+      <c r="C134" s="2" t="inlineStr">
+        <is>
+          <t>الخرج</t>
+        </is>
+      </c>
+      <c r="D134" s="2" t="n">
+        <v>60</v>
+      </c>
+      <c r="E134" s="2" t="inlineStr">
+        <is>
+          <t>د. حسام شلش</t>
+        </is>
+      </c>
+      <c r="F134" s="2" t="inlineStr"/>
+      <c r="G134" s="2" t="inlineStr">
+        <is>
+          <t>نعم</t>
+        </is>
+      </c>
+      <c r="H134" s="2" t="inlineStr">
+        <is>
+          <t>مراجعة فقط</t>
+        </is>
+      </c>
+      <c r="I134" s="3" t="n">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" s="4" t="inlineStr">
         <is>
           <t>الإجمالي</t>
         </is>
       </c>
-      <c r="B127" s="4" t="n"/>
-      <c r="C127" s="4" t="n"/>
-      <c r="D127" s="4" t="n"/>
-      <c r="E127" s="4" t="n"/>
-      <c r="F127" s="4" t="n"/>
-      <c r="G127" s="4" t="n"/>
-      <c r="H127" s="4" t="n"/>
-      <c r="I127" s="5">
-        <f>SUM(I2:I126)</f>
-        <v>20300</v>
+      <c r="B135" s="4" t="n"/>
+      <c r="C135" s="4" t="n"/>
+      <c r="D135" s="4" t="n"/>
+      <c r="E135" s="4" t="n"/>
+      <c r="F135" s="4" t="n"/>
+      <c r="G135" s="4" t="n"/>
+      <c r="H135" s="4" t="n"/>
+      <c r="I135" s="5">
+        <f>SUM(I2:I134)</f>
+        <v>21600</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:I126"/>
+  <autoFilter ref="A1:I134"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Log Oct 14 counts and reviews (pharmacies 24 and 27)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01RnF4y3zxCG7NcjFkMnYdwu
</commit_message>
<xml_diff>
--- a/inventory/jard_log.xlsx
+++ b/inventory/jard_log.xlsx
@@ -10,7 +10,7 @@
     <sheet name="السجل" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'السجل'!$A$1:$I$134</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'السجل'!$A$1:$I$140</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -468,7 +468,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I135"/>
+  <dimension ref="A1:I141"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -5849,25 +5849,267 @@
       </c>
     </row>
     <row r="135">
-      <c r="A135" s="4" t="inlineStr">
+      <c r="A135" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B135" s="2" t="inlineStr">
+        <is>
+          <t>الأربعاء</t>
+        </is>
+      </c>
+      <c r="C135" s="2" t="inlineStr">
+        <is>
+          <t>الخرج</t>
+        </is>
+      </c>
+      <c r="D135" s="2" t="n">
+        <v>24</v>
+      </c>
+      <c r="E135" s="2" t="inlineStr">
+        <is>
+          <t>د. حسام شلش</t>
+        </is>
+      </c>
+      <c r="F135" s="2" t="inlineStr">
+        <is>
+          <t>نعم</t>
+        </is>
+      </c>
+      <c r="G135" s="2" t="inlineStr">
+        <is>
+          <t>نعم</t>
+        </is>
+      </c>
+      <c r="H135" s="2" t="inlineStr">
+        <is>
+          <t>جرد + مراجعة</t>
+        </is>
+      </c>
+      <c r="I135" s="3" t="n">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B136" s="2" t="inlineStr">
+        <is>
+          <t>الأربعاء</t>
+        </is>
+      </c>
+      <c r="C136" s="2" t="inlineStr">
+        <is>
+          <t>الخرج</t>
+        </is>
+      </c>
+      <c r="D136" s="2" t="n">
+        <v>24</v>
+      </c>
+      <c r="E136" s="2" t="inlineStr">
+        <is>
+          <t>د. علي خليفة</t>
+        </is>
+      </c>
+      <c r="F136" s="2" t="inlineStr"/>
+      <c r="G136" s="2" t="inlineStr">
+        <is>
+          <t>نعم</t>
+        </is>
+      </c>
+      <c r="H136" s="2" t="inlineStr">
+        <is>
+          <t>مراجعة فقط</t>
+        </is>
+      </c>
+      <c r="I136" s="3" t="n">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B137" s="2" t="inlineStr">
+        <is>
+          <t>الأربعاء</t>
+        </is>
+      </c>
+      <c r="C137" s="2" t="inlineStr">
+        <is>
+          <t>الخرج</t>
+        </is>
+      </c>
+      <c r="D137" s="2" t="n">
+        <v>24</v>
+      </c>
+      <c r="E137" s="2" t="inlineStr">
+        <is>
+          <t>د. السيد حسن</t>
+        </is>
+      </c>
+      <c r="F137" s="2" t="inlineStr"/>
+      <c r="G137" s="2" t="inlineStr">
+        <is>
+          <t>نعم</t>
+        </is>
+      </c>
+      <c r="H137" s="2" t="inlineStr">
+        <is>
+          <t>مراجعة فقط</t>
+        </is>
+      </c>
+      <c r="I137" s="3" t="n">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B138" s="2" t="inlineStr">
+        <is>
+          <t>الأربعاء</t>
+        </is>
+      </c>
+      <c r="C138" s="2" t="inlineStr">
+        <is>
+          <t>الخرج</t>
+        </is>
+      </c>
+      <c r="D138" s="2" t="n">
+        <v>27</v>
+      </c>
+      <c r="E138" s="2" t="inlineStr">
+        <is>
+          <t>د. حسام شلش</t>
+        </is>
+      </c>
+      <c r="F138" s="2" t="inlineStr">
+        <is>
+          <t>نعم</t>
+        </is>
+      </c>
+      <c r="G138" s="2" t="inlineStr">
+        <is>
+          <t>نعم</t>
+        </is>
+      </c>
+      <c r="H138" s="2" t="inlineStr">
+        <is>
+          <t>جرد + مراجعة</t>
+        </is>
+      </c>
+      <c r="I138" s="3" t="n">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B139" s="2" t="inlineStr">
+        <is>
+          <t>الأربعاء</t>
+        </is>
+      </c>
+      <c r="C139" s="2" t="inlineStr">
+        <is>
+          <t>الخرج</t>
+        </is>
+      </c>
+      <c r="D139" s="2" t="n">
+        <v>27</v>
+      </c>
+      <c r="E139" s="2" t="inlineStr">
+        <is>
+          <t>د. علي خليفة</t>
+        </is>
+      </c>
+      <c r="F139" s="2" t="inlineStr"/>
+      <c r="G139" s="2" t="inlineStr">
+        <is>
+          <t>نعم</t>
+        </is>
+      </c>
+      <c r="H139" s="2" t="inlineStr">
+        <is>
+          <t>مراجعة فقط</t>
+        </is>
+      </c>
+      <c r="I139" s="3" t="n">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B140" s="2" t="inlineStr">
+        <is>
+          <t>الأربعاء</t>
+        </is>
+      </c>
+      <c r="C140" s="2" t="inlineStr">
+        <is>
+          <t>الخرج</t>
+        </is>
+      </c>
+      <c r="D140" s="2" t="n">
+        <v>27</v>
+      </c>
+      <c r="E140" s="2" t="inlineStr">
+        <is>
+          <t>د. السيد حسن</t>
+        </is>
+      </c>
+      <c r="F140" s="2" t="inlineStr"/>
+      <c r="G140" s="2" t="inlineStr">
+        <is>
+          <t>نعم</t>
+        </is>
+      </c>
+      <c r="H140" s="2" t="inlineStr">
+        <is>
+          <t>مراجعة فقط</t>
+        </is>
+      </c>
+      <c r="I140" s="3" t="n">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" s="4" t="inlineStr">
         <is>
           <t>الإجمالي</t>
         </is>
       </c>
-      <c r="B135" s="4" t="n"/>
-      <c r="C135" s="4" t="n"/>
-      <c r="D135" s="4" t="n"/>
-      <c r="E135" s="4" t="n"/>
-      <c r="F135" s="4" t="n"/>
-      <c r="G135" s="4" t="n"/>
-      <c r="H135" s="4" t="n"/>
-      <c r="I135" s="5">
-        <f>SUM(I2:I134)</f>
-        <v>21600</v>
+      <c r="B141" s="4" t="n"/>
+      <c r="C141" s="4" t="n"/>
+      <c r="D141" s="4" t="n"/>
+      <c r="E141" s="4" t="n"/>
+      <c r="F141" s="4" t="n"/>
+      <c r="G141" s="4" t="n"/>
+      <c r="H141" s="4" t="n"/>
+      <c r="I141" s="5">
+        <f>SUM(I2:I140)</f>
+        <v>22600</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:I134"/>
+  <autoFilter ref="A1:I140"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Log Oct 15 counts and reviews (pharmacies 11 and 40)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01RnF4y3zxCG7NcjFkMnYdwu
</commit_message>
<xml_diff>
--- a/inventory/jard_log.xlsx
+++ b/inventory/jard_log.xlsx
@@ -10,7 +10,7 @@
     <sheet name="السجل" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'السجل'!$A$1:$I$140</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'السجل'!$A$1:$I$146</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -468,7 +468,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I141"/>
+  <dimension ref="A1:I147"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -6091,25 +6091,267 @@
       </c>
     </row>
     <row r="141">
-      <c r="A141" s="4" t="inlineStr">
+      <c r="A141" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="B141" s="2" t="inlineStr">
+        <is>
+          <t>الخميس</t>
+        </is>
+      </c>
+      <c r="C141" s="2" t="inlineStr">
+        <is>
+          <t>الخرج</t>
+        </is>
+      </c>
+      <c r="D141" s="2" t="n">
+        <v>11</v>
+      </c>
+      <c r="E141" s="2" t="inlineStr">
+        <is>
+          <t>د. علي خليفة</t>
+        </is>
+      </c>
+      <c r="F141" s="2" t="inlineStr">
+        <is>
+          <t>نعم</t>
+        </is>
+      </c>
+      <c r="G141" s="2" t="inlineStr">
+        <is>
+          <t>نعم</t>
+        </is>
+      </c>
+      <c r="H141" s="2" t="inlineStr">
+        <is>
+          <t>جرد + مراجعة</t>
+        </is>
+      </c>
+      <c r="I141" s="3" t="n">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="B142" s="2" t="inlineStr">
+        <is>
+          <t>الخميس</t>
+        </is>
+      </c>
+      <c r="C142" s="2" t="inlineStr">
+        <is>
+          <t>الخرج</t>
+        </is>
+      </c>
+      <c r="D142" s="2" t="n">
+        <v>11</v>
+      </c>
+      <c r="E142" s="2" t="inlineStr">
+        <is>
+          <t>د. حسام شلش</t>
+        </is>
+      </c>
+      <c r="F142" s="2" t="inlineStr"/>
+      <c r="G142" s="2" t="inlineStr">
+        <is>
+          <t>نعم</t>
+        </is>
+      </c>
+      <c r="H142" s="2" t="inlineStr">
+        <is>
+          <t>مراجعة فقط</t>
+        </is>
+      </c>
+      <c r="I142" s="3" t="n">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="B143" s="2" t="inlineStr">
+        <is>
+          <t>الخميس</t>
+        </is>
+      </c>
+      <c r="C143" s="2" t="inlineStr">
+        <is>
+          <t>الخرج</t>
+        </is>
+      </c>
+      <c r="D143" s="2" t="n">
+        <v>11</v>
+      </c>
+      <c r="E143" s="2" t="inlineStr">
+        <is>
+          <t>د. السيد حسن</t>
+        </is>
+      </c>
+      <c r="F143" s="2" t="inlineStr"/>
+      <c r="G143" s="2" t="inlineStr">
+        <is>
+          <t>نعم</t>
+        </is>
+      </c>
+      <c r="H143" s="2" t="inlineStr">
+        <is>
+          <t>مراجعة فقط</t>
+        </is>
+      </c>
+      <c r="I143" s="3" t="n">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="B144" s="2" t="inlineStr">
+        <is>
+          <t>الخميس</t>
+        </is>
+      </c>
+      <c r="C144" s="2" t="inlineStr">
+        <is>
+          <t>الخرج</t>
+        </is>
+      </c>
+      <c r="D144" s="2" t="n">
+        <v>40</v>
+      </c>
+      <c r="E144" s="2" t="inlineStr">
+        <is>
+          <t>د. علي خليفة</t>
+        </is>
+      </c>
+      <c r="F144" s="2" t="inlineStr">
+        <is>
+          <t>نعم</t>
+        </is>
+      </c>
+      <c r="G144" s="2" t="inlineStr">
+        <is>
+          <t>نعم</t>
+        </is>
+      </c>
+      <c r="H144" s="2" t="inlineStr">
+        <is>
+          <t>جرد + مراجعة</t>
+        </is>
+      </c>
+      <c r="I144" s="3" t="n">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="B145" s="2" t="inlineStr">
+        <is>
+          <t>الخميس</t>
+        </is>
+      </c>
+      <c r="C145" s="2" t="inlineStr">
+        <is>
+          <t>الخرج</t>
+        </is>
+      </c>
+      <c r="D145" s="2" t="n">
+        <v>40</v>
+      </c>
+      <c r="E145" s="2" t="inlineStr">
+        <is>
+          <t>د. حسام شلش</t>
+        </is>
+      </c>
+      <c r="F145" s="2" t="inlineStr"/>
+      <c r="G145" s="2" t="inlineStr">
+        <is>
+          <t>نعم</t>
+        </is>
+      </c>
+      <c r="H145" s="2" t="inlineStr">
+        <is>
+          <t>مراجعة فقط</t>
+        </is>
+      </c>
+      <c r="I145" s="3" t="n">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="B146" s="2" t="inlineStr">
+        <is>
+          <t>الخميس</t>
+        </is>
+      </c>
+      <c r="C146" s="2" t="inlineStr">
+        <is>
+          <t>الخرج</t>
+        </is>
+      </c>
+      <c r="D146" s="2" t="n">
+        <v>40</v>
+      </c>
+      <c r="E146" s="2" t="inlineStr">
+        <is>
+          <t>د. السيد حسن</t>
+        </is>
+      </c>
+      <c r="F146" s="2" t="inlineStr"/>
+      <c r="G146" s="2" t="inlineStr">
+        <is>
+          <t>نعم</t>
+        </is>
+      </c>
+      <c r="H146" s="2" t="inlineStr">
+        <is>
+          <t>مراجعة فقط</t>
+        </is>
+      </c>
+      <c r="I146" s="3" t="n">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" s="4" t="inlineStr">
         <is>
           <t>الإجمالي</t>
         </is>
       </c>
-      <c r="B141" s="4" t="n"/>
-      <c r="C141" s="4" t="n"/>
-      <c r="D141" s="4" t="n"/>
-      <c r="E141" s="4" t="n"/>
-      <c r="F141" s="4" t="n"/>
-      <c r="G141" s="4" t="n"/>
-      <c r="H141" s="4" t="n"/>
-      <c r="I141" s="5">
-        <f>SUM(I2:I140)</f>
-        <v>22600</v>
+      <c r="B147" s="4" t="n"/>
+      <c r="C147" s="4" t="n"/>
+      <c r="D147" s="4" t="n"/>
+      <c r="E147" s="4" t="n"/>
+      <c r="F147" s="4" t="n"/>
+      <c r="G147" s="4" t="n"/>
+      <c r="H147" s="4" t="n"/>
+      <c r="I147" s="5">
+        <f>SUM(I2:I146)</f>
+        <v>23600</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:I140"/>
+  <autoFilter ref="A1:I146"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Log Oct 16 count and reviews (pharmacy 18)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01RnF4y3zxCG7NcjFkMnYdwu
</commit_message>
<xml_diff>
--- a/inventory/jard_log.xlsx
+++ b/inventory/jard_log.xlsx
@@ -10,7 +10,7 @@
     <sheet name="السجل" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'السجل'!$A$1:$I$146</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'السجل'!$A$1:$I$150</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -468,7 +468,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I147"/>
+  <dimension ref="A1:I151"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -6333,25 +6333,185 @@
       </c>
     </row>
     <row r="147">
-      <c r="A147" s="4" t="inlineStr">
+      <c r="A147" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="B147" s="2" t="inlineStr">
+        <is>
+          <t>الجمعة</t>
+        </is>
+      </c>
+      <c r="C147" s="2" t="inlineStr">
+        <is>
+          <t>الخرج</t>
+        </is>
+      </c>
+      <c r="D147" s="2" t="n">
+        <v>18</v>
+      </c>
+      <c r="E147" s="2" t="inlineStr">
+        <is>
+          <t>د. حسام شلش</t>
+        </is>
+      </c>
+      <c r="F147" s="2" t="inlineStr">
+        <is>
+          <t>نعم</t>
+        </is>
+      </c>
+      <c r="G147" s="2" t="inlineStr">
+        <is>
+          <t>نعم</t>
+        </is>
+      </c>
+      <c r="H147" s="2" t="inlineStr">
+        <is>
+          <t>جرد + مراجعة</t>
+        </is>
+      </c>
+      <c r="I147" s="3" t="n">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="B148" s="2" t="inlineStr">
+        <is>
+          <t>الجمعة</t>
+        </is>
+      </c>
+      <c r="C148" s="2" t="inlineStr">
+        <is>
+          <t>الخرج</t>
+        </is>
+      </c>
+      <c r="D148" s="2" t="n">
+        <v>18</v>
+      </c>
+      <c r="E148" s="2" t="inlineStr">
+        <is>
+          <t>د. علي خليفة</t>
+        </is>
+      </c>
+      <c r="F148" s="2" t="inlineStr"/>
+      <c r="G148" s="2" t="inlineStr">
+        <is>
+          <t>نعم</t>
+        </is>
+      </c>
+      <c r="H148" s="2" t="inlineStr">
+        <is>
+          <t>مراجعة فقط</t>
+        </is>
+      </c>
+      <c r="I148" s="3" t="n">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="B149" s="2" t="inlineStr">
+        <is>
+          <t>الجمعة</t>
+        </is>
+      </c>
+      <c r="C149" s="2" t="inlineStr">
+        <is>
+          <t>الخرج</t>
+        </is>
+      </c>
+      <c r="D149" s="2" t="n">
+        <v>18</v>
+      </c>
+      <c r="E149" s="2" t="inlineStr">
+        <is>
+          <t>د. الحسن الغنيمي</t>
+        </is>
+      </c>
+      <c r="F149" s="2" t="inlineStr"/>
+      <c r="G149" s="2" t="inlineStr">
+        <is>
+          <t>نعم</t>
+        </is>
+      </c>
+      <c r="H149" s="2" t="inlineStr">
+        <is>
+          <t>مراجعة فقط</t>
+        </is>
+      </c>
+      <c r="I149" s="3" t="n">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="B150" s="2" t="inlineStr">
+        <is>
+          <t>الجمعة</t>
+        </is>
+      </c>
+      <c r="C150" s="2" t="inlineStr">
+        <is>
+          <t>الخرج</t>
+        </is>
+      </c>
+      <c r="D150" s="2" t="n">
+        <v>18</v>
+      </c>
+      <c r="E150" s="2" t="inlineStr">
+        <is>
+          <t>د. محمد فؤاد</t>
+        </is>
+      </c>
+      <c r="F150" s="2" t="inlineStr"/>
+      <c r="G150" s="2" t="inlineStr">
+        <is>
+          <t>نعم</t>
+        </is>
+      </c>
+      <c r="H150" s="2" t="inlineStr">
+        <is>
+          <t>مراجعة فقط</t>
+        </is>
+      </c>
+      <c r="I150" s="3" t="n">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" s="4" t="inlineStr">
         <is>
           <t>الإجمالي</t>
         </is>
       </c>
-      <c r="B147" s="4" t="n"/>
-      <c r="C147" s="4" t="n"/>
-      <c r="D147" s="4" t="n"/>
-      <c r="E147" s="4" t="n"/>
-      <c r="F147" s="4" t="n"/>
-      <c r="G147" s="4" t="n"/>
-      <c r="H147" s="4" t="n"/>
-      <c r="I147" s="5">
-        <f>SUM(I2:I146)</f>
-        <v>23600</v>
+      <c r="B151" s="4" t="n"/>
+      <c r="C151" s="4" t="n"/>
+      <c r="D151" s="4" t="n"/>
+      <c r="E151" s="4" t="n"/>
+      <c r="F151" s="4" t="n"/>
+      <c r="G151" s="4" t="n"/>
+      <c r="H151" s="4" t="n"/>
+      <c r="I151" s="5">
+        <f>SUM(I2:I150)</f>
+        <v>24250</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:I146"/>
+  <autoFilter ref="A1:I150"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Log Oct 17 count and reviews (pharmacy 19)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01RnF4y3zxCG7NcjFkMnYdwu
</commit_message>
<xml_diff>
--- a/inventory/jard_log.xlsx
+++ b/inventory/jard_log.xlsx
@@ -10,7 +10,7 @@
     <sheet name="السجل" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'السجل'!$A$1:$I$150</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'السجل'!$A$1:$I$153</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -468,7 +468,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I151"/>
+  <dimension ref="A1:I154"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -6493,25 +6493,146 @@
       </c>
     </row>
     <row r="151">
-      <c r="A151" s="4" t="inlineStr">
+      <c r="A151" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-17</t>
+        </is>
+      </c>
+      <c r="B151" s="2" t="inlineStr">
+        <is>
+          <t>السبت</t>
+        </is>
+      </c>
+      <c r="C151" s="2" t="inlineStr">
+        <is>
+          <t>الخرج</t>
+        </is>
+      </c>
+      <c r="D151" s="2" t="n">
+        <v>19</v>
+      </c>
+      <c r="E151" s="2" t="inlineStr">
+        <is>
+          <t>د. علي خليفة</t>
+        </is>
+      </c>
+      <c r="F151" s="2" t="inlineStr">
+        <is>
+          <t>نعم</t>
+        </is>
+      </c>
+      <c r="G151" s="2" t="inlineStr">
+        <is>
+          <t>نعم</t>
+        </is>
+      </c>
+      <c r="H151" s="2" t="inlineStr">
+        <is>
+          <t>جرد + مراجعة</t>
+        </is>
+      </c>
+      <c r="I151" s="3" t="n">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-17</t>
+        </is>
+      </c>
+      <c r="B152" s="2" t="inlineStr">
+        <is>
+          <t>السبت</t>
+        </is>
+      </c>
+      <c r="C152" s="2" t="inlineStr">
+        <is>
+          <t>الخرج</t>
+        </is>
+      </c>
+      <c r="D152" s="2" t="n">
+        <v>19</v>
+      </c>
+      <c r="E152" s="2" t="inlineStr">
+        <is>
+          <t>د. السيد حسن</t>
+        </is>
+      </c>
+      <c r="F152" s="2" t="inlineStr"/>
+      <c r="G152" s="2" t="inlineStr">
+        <is>
+          <t>نعم</t>
+        </is>
+      </c>
+      <c r="H152" s="2" t="inlineStr">
+        <is>
+          <t>مراجعة فقط</t>
+        </is>
+      </c>
+      <c r="I152" s="3" t="n">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-17</t>
+        </is>
+      </c>
+      <c r="B153" s="2" t="inlineStr">
+        <is>
+          <t>السبت</t>
+        </is>
+      </c>
+      <c r="C153" s="2" t="inlineStr">
+        <is>
+          <t>الخرج</t>
+        </is>
+      </c>
+      <c r="D153" s="2" t="n">
+        <v>19</v>
+      </c>
+      <c r="E153" s="2" t="inlineStr">
+        <is>
+          <t>د. حسام شلش</t>
+        </is>
+      </c>
+      <c r="F153" s="2" t="inlineStr"/>
+      <c r="G153" s="2" t="inlineStr">
+        <is>
+          <t>نعم</t>
+        </is>
+      </c>
+      <c r="H153" s="2" t="inlineStr">
+        <is>
+          <t>مراجعة فقط</t>
+        </is>
+      </c>
+      <c r="I153" s="3" t="n">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" s="4" t="inlineStr">
         <is>
           <t>الإجمالي</t>
         </is>
       </c>
-      <c r="B151" s="4" t="n"/>
-      <c r="C151" s="4" t="n"/>
-      <c r="D151" s="4" t="n"/>
-      <c r="E151" s="4" t="n"/>
-      <c r="F151" s="4" t="n"/>
-      <c r="G151" s="4" t="n"/>
-      <c r="H151" s="4" t="n"/>
-      <c r="I151" s="5">
-        <f>SUM(I2:I150)</f>
-        <v>24250</v>
+      <c r="B154" s="4" t="n"/>
+      <c r="C154" s="4" t="n"/>
+      <c r="D154" s="4" t="n"/>
+      <c r="E154" s="4" t="n"/>
+      <c r="F154" s="4" t="n"/>
+      <c r="G154" s="4" t="n"/>
+      <c r="H154" s="4" t="n"/>
+      <c r="I154" s="5">
+        <f>SUM(I2:I153)</f>
+        <v>24750</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:I150"/>
+  <autoFilter ref="A1:I153"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Log Oct 18 count and reviews (pharmacy 14)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01RnF4y3zxCG7NcjFkMnYdwu
</commit_message>
<xml_diff>
--- a/inventory/jard_log.xlsx
+++ b/inventory/jard_log.xlsx
@@ -10,7 +10,7 @@
     <sheet name="السجل" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'السجل'!$A$1:$I$153</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'السجل'!$A$1:$I$156</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -468,7 +468,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I154"/>
+  <dimension ref="A1:I157"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -6614,25 +6614,146 @@
       </c>
     </row>
     <row r="154">
-      <c r="A154" s="4" t="inlineStr">
+      <c r="A154" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-18</t>
+        </is>
+      </c>
+      <c r="B154" s="2" t="inlineStr">
+        <is>
+          <t>الأحد</t>
+        </is>
+      </c>
+      <c r="C154" s="2" t="inlineStr">
+        <is>
+          <t>الخرج</t>
+        </is>
+      </c>
+      <c r="D154" s="2" t="n">
+        <v>14</v>
+      </c>
+      <c r="E154" s="2" t="inlineStr">
+        <is>
+          <t>د. حسام شلش</t>
+        </is>
+      </c>
+      <c r="F154" s="2" t="inlineStr">
+        <is>
+          <t>نعم</t>
+        </is>
+      </c>
+      <c r="G154" s="2" t="inlineStr">
+        <is>
+          <t>نعم</t>
+        </is>
+      </c>
+      <c r="H154" s="2" t="inlineStr">
+        <is>
+          <t>جرد + مراجعة</t>
+        </is>
+      </c>
+      <c r="I154" s="3" t="n">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-18</t>
+        </is>
+      </c>
+      <c r="B155" s="2" t="inlineStr">
+        <is>
+          <t>الأحد</t>
+        </is>
+      </c>
+      <c r="C155" s="2" t="inlineStr">
+        <is>
+          <t>الخرج</t>
+        </is>
+      </c>
+      <c r="D155" s="2" t="n">
+        <v>14</v>
+      </c>
+      <c r="E155" s="2" t="inlineStr">
+        <is>
+          <t>د. علي خليفة</t>
+        </is>
+      </c>
+      <c r="F155" s="2" t="inlineStr"/>
+      <c r="G155" s="2" t="inlineStr">
+        <is>
+          <t>نعم</t>
+        </is>
+      </c>
+      <c r="H155" s="2" t="inlineStr">
+        <is>
+          <t>مراجعة فقط</t>
+        </is>
+      </c>
+      <c r="I155" s="3" t="n">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-18</t>
+        </is>
+      </c>
+      <c r="B156" s="2" t="inlineStr">
+        <is>
+          <t>الأحد</t>
+        </is>
+      </c>
+      <c r="C156" s="2" t="inlineStr">
+        <is>
+          <t>الخرج</t>
+        </is>
+      </c>
+      <c r="D156" s="2" t="n">
+        <v>14</v>
+      </c>
+      <c r="E156" s="2" t="inlineStr">
+        <is>
+          <t>د. السيد حسن</t>
+        </is>
+      </c>
+      <c r="F156" s="2" t="inlineStr"/>
+      <c r="G156" s="2" t="inlineStr">
+        <is>
+          <t>نعم</t>
+        </is>
+      </c>
+      <c r="H156" s="2" t="inlineStr">
+        <is>
+          <t>مراجعة فقط</t>
+        </is>
+      </c>
+      <c r="I156" s="3" t="n">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" s="4" t="inlineStr">
         <is>
           <t>الإجمالي</t>
         </is>
       </c>
-      <c r="B154" s="4" t="n"/>
-      <c r="C154" s="4" t="n"/>
-      <c r="D154" s="4" t="n"/>
-      <c r="E154" s="4" t="n"/>
-      <c r="F154" s="4" t="n"/>
-      <c r="G154" s="4" t="n"/>
-      <c r="H154" s="4" t="n"/>
-      <c r="I154" s="5">
-        <f>SUM(I2:I153)</f>
-        <v>24750</v>
+      <c r="B157" s="4" t="n"/>
+      <c r="C157" s="4" t="n"/>
+      <c r="D157" s="4" t="n"/>
+      <c r="E157" s="4" t="n"/>
+      <c r="F157" s="4" t="n"/>
+      <c r="G157" s="4" t="n"/>
+      <c r="H157" s="4" t="n"/>
+      <c r="I157" s="5">
+        <f>SUM(I2:I156)</f>
+        <v>25250</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:I153"/>
+  <autoFilter ref="A1:I156"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Log Oct 19 counts and reviews (pharmacies 42 and 44)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01RnF4y3zxCG7NcjFkMnYdwu
</commit_message>
<xml_diff>
--- a/inventory/jard_log.xlsx
+++ b/inventory/jard_log.xlsx
@@ -10,7 +10,7 @@
     <sheet name="السجل" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'السجل'!$A$1:$I$156</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'السجل'!$A$1:$I$162</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -468,7 +468,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I157"/>
+  <dimension ref="A1:I163"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -6735,25 +6735,267 @@
       </c>
     </row>
     <row r="157">
-      <c r="A157" s="4" t="inlineStr">
+      <c r="A157" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
+      <c r="B157" s="2" t="inlineStr">
+        <is>
+          <t>الاثنين</t>
+        </is>
+      </c>
+      <c r="C157" s="2" t="inlineStr">
+        <is>
+          <t>الرياض</t>
+        </is>
+      </c>
+      <c r="D157" s="2" t="n">
+        <v>42</v>
+      </c>
+      <c r="E157" s="2" t="inlineStr">
+        <is>
+          <t>د. علي خليفة</t>
+        </is>
+      </c>
+      <c r="F157" s="2" t="inlineStr">
+        <is>
+          <t>نعم</t>
+        </is>
+      </c>
+      <c r="G157" s="2" t="inlineStr">
+        <is>
+          <t>نعم</t>
+        </is>
+      </c>
+      <c r="H157" s="2" t="inlineStr">
+        <is>
+          <t>جرد + مراجعة</t>
+        </is>
+      </c>
+      <c r="I157" s="3" t="n">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
+      <c r="B158" s="2" t="inlineStr">
+        <is>
+          <t>الاثنين</t>
+        </is>
+      </c>
+      <c r="C158" s="2" t="inlineStr">
+        <is>
+          <t>الرياض</t>
+        </is>
+      </c>
+      <c r="D158" s="2" t="n">
+        <v>42</v>
+      </c>
+      <c r="E158" s="2" t="inlineStr">
+        <is>
+          <t>د. حسام شلش</t>
+        </is>
+      </c>
+      <c r="F158" s="2" t="inlineStr"/>
+      <c r="G158" s="2" t="inlineStr">
+        <is>
+          <t>نعم</t>
+        </is>
+      </c>
+      <c r="H158" s="2" t="inlineStr">
+        <is>
+          <t>مراجعة فقط</t>
+        </is>
+      </c>
+      <c r="I158" s="3" t="n">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
+      <c r="B159" s="2" t="inlineStr">
+        <is>
+          <t>الاثنين</t>
+        </is>
+      </c>
+      <c r="C159" s="2" t="inlineStr">
+        <is>
+          <t>الرياض</t>
+        </is>
+      </c>
+      <c r="D159" s="2" t="n">
+        <v>42</v>
+      </c>
+      <c r="E159" s="2" t="inlineStr">
+        <is>
+          <t>د. السيد حسن</t>
+        </is>
+      </c>
+      <c r="F159" s="2" t="inlineStr"/>
+      <c r="G159" s="2" t="inlineStr">
+        <is>
+          <t>نعم</t>
+        </is>
+      </c>
+      <c r="H159" s="2" t="inlineStr">
+        <is>
+          <t>مراجعة فقط</t>
+        </is>
+      </c>
+      <c r="I159" s="3" t="n">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
+      <c r="B160" s="2" t="inlineStr">
+        <is>
+          <t>الاثنين</t>
+        </is>
+      </c>
+      <c r="C160" s="2" t="inlineStr">
+        <is>
+          <t>الرياض</t>
+        </is>
+      </c>
+      <c r="D160" s="2" t="n">
+        <v>44</v>
+      </c>
+      <c r="E160" s="2" t="inlineStr">
+        <is>
+          <t>د. علي خليفة</t>
+        </is>
+      </c>
+      <c r="F160" s="2" t="inlineStr">
+        <is>
+          <t>نعم</t>
+        </is>
+      </c>
+      <c r="G160" s="2" t="inlineStr">
+        <is>
+          <t>نعم</t>
+        </is>
+      </c>
+      <c r="H160" s="2" t="inlineStr">
+        <is>
+          <t>جرد + مراجعة</t>
+        </is>
+      </c>
+      <c r="I160" s="3" t="n">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
+      <c r="B161" s="2" t="inlineStr">
+        <is>
+          <t>الاثنين</t>
+        </is>
+      </c>
+      <c r="C161" s="2" t="inlineStr">
+        <is>
+          <t>الرياض</t>
+        </is>
+      </c>
+      <c r="D161" s="2" t="n">
+        <v>44</v>
+      </c>
+      <c r="E161" s="2" t="inlineStr">
+        <is>
+          <t>د. حسام شلش</t>
+        </is>
+      </c>
+      <c r="F161" s="2" t="inlineStr"/>
+      <c r="G161" s="2" t="inlineStr">
+        <is>
+          <t>نعم</t>
+        </is>
+      </c>
+      <c r="H161" s="2" t="inlineStr">
+        <is>
+          <t>مراجعة فقط</t>
+        </is>
+      </c>
+      <c r="I161" s="3" t="n">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
+      <c r="B162" s="2" t="inlineStr">
+        <is>
+          <t>الاثنين</t>
+        </is>
+      </c>
+      <c r="C162" s="2" t="inlineStr">
+        <is>
+          <t>الرياض</t>
+        </is>
+      </c>
+      <c r="D162" s="2" t="n">
+        <v>44</v>
+      </c>
+      <c r="E162" s="2" t="inlineStr">
+        <is>
+          <t>د. السيد حسن</t>
+        </is>
+      </c>
+      <c r="F162" s="2" t="inlineStr"/>
+      <c r="G162" s="2" t="inlineStr">
+        <is>
+          <t>نعم</t>
+        </is>
+      </c>
+      <c r="H162" s="2" t="inlineStr">
+        <is>
+          <t>مراجعة فقط</t>
+        </is>
+      </c>
+      <c r="I162" s="3" t="n">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" s="4" t="inlineStr">
         <is>
           <t>الإجمالي</t>
         </is>
       </c>
-      <c r="B157" s="4" t="n"/>
-      <c r="C157" s="4" t="n"/>
-      <c r="D157" s="4" t="n"/>
-      <c r="E157" s="4" t="n"/>
-      <c r="F157" s="4" t="n"/>
-      <c r="G157" s="4" t="n"/>
-      <c r="H157" s="4" t="n"/>
-      <c r="I157" s="5">
-        <f>SUM(I2:I156)</f>
-        <v>25250</v>
+      <c r="B163" s="4" t="n"/>
+      <c r="C163" s="4" t="n"/>
+      <c r="D163" s="4" t="n"/>
+      <c r="E163" s="4" t="n"/>
+      <c r="F163" s="4" t="n"/>
+      <c r="G163" s="4" t="n"/>
+      <c r="H163" s="4" t="n"/>
+      <c r="I163" s="5">
+        <f>SUM(I2:I162)</f>
+        <v>26250</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:I156"/>
+  <autoFilter ref="A1:I162"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Log Oct 20 counts and reviews (pharmacies 43 and 45)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01RnF4y3zxCG7NcjFkMnYdwu
</commit_message>
<xml_diff>
--- a/inventory/jard_log.xlsx
+++ b/inventory/jard_log.xlsx
@@ -10,7 +10,7 @@
     <sheet name="السجل" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'السجل'!$A$1:$I$162</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'السجل'!$A$1:$I$166</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -468,7 +468,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I163"/>
+  <dimension ref="A1:I167"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -6977,25 +6977,189 @@
       </c>
     </row>
     <row r="163">
-      <c r="A163" s="4" t="inlineStr">
+      <c r="A163" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="B163" s="2" t="inlineStr">
+        <is>
+          <t>الثلاثاء</t>
+        </is>
+      </c>
+      <c r="C163" s="2" t="inlineStr">
+        <is>
+          <t>الرياض</t>
+        </is>
+      </c>
+      <c r="D163" s="2" t="n">
+        <v>43</v>
+      </c>
+      <c r="E163" s="2" t="inlineStr">
+        <is>
+          <t>د. حسام شلش</t>
+        </is>
+      </c>
+      <c r="F163" s="2" t="inlineStr">
+        <is>
+          <t>نعم</t>
+        </is>
+      </c>
+      <c r="G163" s="2" t="inlineStr">
+        <is>
+          <t>نعم</t>
+        </is>
+      </c>
+      <c r="H163" s="2" t="inlineStr">
+        <is>
+          <t>جرد + مراجعة</t>
+        </is>
+      </c>
+      <c r="I163" s="3" t="n">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="B164" s="2" t="inlineStr">
+        <is>
+          <t>الثلاثاء</t>
+        </is>
+      </c>
+      <c r="C164" s="2" t="inlineStr">
+        <is>
+          <t>الرياض</t>
+        </is>
+      </c>
+      <c r="D164" s="2" t="n">
+        <v>43</v>
+      </c>
+      <c r="E164" s="2" t="inlineStr">
+        <is>
+          <t>د. السيد حسن</t>
+        </is>
+      </c>
+      <c r="F164" s="2" t="inlineStr"/>
+      <c r="G164" s="2" t="inlineStr">
+        <is>
+          <t>نعم</t>
+        </is>
+      </c>
+      <c r="H164" s="2" t="inlineStr">
+        <is>
+          <t>مراجعة فقط</t>
+        </is>
+      </c>
+      <c r="I164" s="3" t="n">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="B165" s="2" t="inlineStr">
+        <is>
+          <t>الثلاثاء</t>
+        </is>
+      </c>
+      <c r="C165" s="2" t="inlineStr">
+        <is>
+          <t>الرياض</t>
+        </is>
+      </c>
+      <c r="D165" s="2" t="n">
+        <v>45</v>
+      </c>
+      <c r="E165" s="2" t="inlineStr">
+        <is>
+          <t>د. حسام شلش</t>
+        </is>
+      </c>
+      <c r="F165" s="2" t="inlineStr">
+        <is>
+          <t>نعم</t>
+        </is>
+      </c>
+      <c r="G165" s="2" t="inlineStr">
+        <is>
+          <t>نعم</t>
+        </is>
+      </c>
+      <c r="H165" s="2" t="inlineStr">
+        <is>
+          <t>جرد + مراجعة</t>
+        </is>
+      </c>
+      <c r="I165" s="3" t="n">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="B166" s="2" t="inlineStr">
+        <is>
+          <t>الثلاثاء</t>
+        </is>
+      </c>
+      <c r="C166" s="2" t="inlineStr">
+        <is>
+          <t>الرياض</t>
+        </is>
+      </c>
+      <c r="D166" s="2" t="n">
+        <v>45</v>
+      </c>
+      <c r="E166" s="2" t="inlineStr">
+        <is>
+          <t>د. السيد حسن</t>
+        </is>
+      </c>
+      <c r="F166" s="2" t="inlineStr"/>
+      <c r="G166" s="2" t="inlineStr">
+        <is>
+          <t>نعم</t>
+        </is>
+      </c>
+      <c r="H166" s="2" t="inlineStr">
+        <is>
+          <t>مراجعة فقط</t>
+        </is>
+      </c>
+      <c r="I166" s="3" t="n">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167" s="4" t="inlineStr">
         <is>
           <t>الإجمالي</t>
         </is>
       </c>
-      <c r="B163" s="4" t="n"/>
-      <c r="C163" s="4" t="n"/>
-      <c r="D163" s="4" t="n"/>
-      <c r="E163" s="4" t="n"/>
-      <c r="F163" s="4" t="n"/>
-      <c r="G163" s="4" t="n"/>
-      <c r="H163" s="4" t="n"/>
-      <c r="I163" s="5">
-        <f>SUM(I2:I162)</f>
-        <v>26250</v>
+      <c r="B167" s="4" t="n"/>
+      <c r="C167" s="4" t="n"/>
+      <c r="D167" s="4" t="n"/>
+      <c r="E167" s="4" t="n"/>
+      <c r="F167" s="4" t="n"/>
+      <c r="G167" s="4" t="n"/>
+      <c r="H167" s="4" t="n"/>
+      <c r="I167" s="5">
+        <f>SUM(I2:I166)</f>
+        <v>26950</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:I162"/>
+  <autoFilter ref="A1:I166"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Log Oct 21 counts and reviews (pharmacies 23 and 58)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01RnF4y3zxCG7NcjFkMnYdwu
</commit_message>
<xml_diff>
--- a/inventory/jard_log.xlsx
+++ b/inventory/jard_log.xlsx
@@ -10,7 +10,7 @@
     <sheet name="السجل" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'السجل'!$A$1:$I$166</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'السجل'!$A$1:$I$172</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -468,7 +468,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I167"/>
+  <dimension ref="A1:I173"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -7141,25 +7141,267 @@
       </c>
     </row>
     <row r="167">
-      <c r="A167" s="4" t="inlineStr">
+      <c r="A167" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="B167" s="2" t="inlineStr">
+        <is>
+          <t>الأربعاء</t>
+        </is>
+      </c>
+      <c r="C167" s="2" t="inlineStr">
+        <is>
+          <t>الرياض</t>
+        </is>
+      </c>
+      <c r="D167" s="2" t="n">
+        <v>23</v>
+      </c>
+      <c r="E167" s="2" t="inlineStr">
+        <is>
+          <t>د. علي خليفة</t>
+        </is>
+      </c>
+      <c r="F167" s="2" t="inlineStr">
+        <is>
+          <t>نعم</t>
+        </is>
+      </c>
+      <c r="G167" s="2" t="inlineStr">
+        <is>
+          <t>نعم</t>
+        </is>
+      </c>
+      <c r="H167" s="2" t="inlineStr">
+        <is>
+          <t>جرد + مراجعة</t>
+        </is>
+      </c>
+      <c r="I167" s="3" t="n">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="168">
+      <c r="A168" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="B168" s="2" t="inlineStr">
+        <is>
+          <t>الأربعاء</t>
+        </is>
+      </c>
+      <c r="C168" s="2" t="inlineStr">
+        <is>
+          <t>الرياض</t>
+        </is>
+      </c>
+      <c r="D168" s="2" t="n">
+        <v>23</v>
+      </c>
+      <c r="E168" s="2" t="inlineStr">
+        <is>
+          <t>د. حسام شلش</t>
+        </is>
+      </c>
+      <c r="F168" s="2" t="inlineStr"/>
+      <c r="G168" s="2" t="inlineStr">
+        <is>
+          <t>نعم</t>
+        </is>
+      </c>
+      <c r="H168" s="2" t="inlineStr">
+        <is>
+          <t>مراجعة فقط</t>
+        </is>
+      </c>
+      <c r="I168" s="3" t="n">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="169">
+      <c r="A169" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="B169" s="2" t="inlineStr">
+        <is>
+          <t>الأربعاء</t>
+        </is>
+      </c>
+      <c r="C169" s="2" t="inlineStr">
+        <is>
+          <t>الرياض</t>
+        </is>
+      </c>
+      <c r="D169" s="2" t="n">
+        <v>23</v>
+      </c>
+      <c r="E169" s="2" t="inlineStr">
+        <is>
+          <t>د. السيد حسن</t>
+        </is>
+      </c>
+      <c r="F169" s="2" t="inlineStr"/>
+      <c r="G169" s="2" t="inlineStr">
+        <is>
+          <t>نعم</t>
+        </is>
+      </c>
+      <c r="H169" s="2" t="inlineStr">
+        <is>
+          <t>مراجعة فقط</t>
+        </is>
+      </c>
+      <c r="I169" s="3" t="n">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="170">
+      <c r="A170" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="B170" s="2" t="inlineStr">
+        <is>
+          <t>الأربعاء</t>
+        </is>
+      </c>
+      <c r="C170" s="2" t="inlineStr">
+        <is>
+          <t>الرياض</t>
+        </is>
+      </c>
+      <c r="D170" s="2" t="n">
+        <v>58</v>
+      </c>
+      <c r="E170" s="2" t="inlineStr">
+        <is>
+          <t>د. علي خليفة</t>
+        </is>
+      </c>
+      <c r="F170" s="2" t="inlineStr">
+        <is>
+          <t>نعم</t>
+        </is>
+      </c>
+      <c r="G170" s="2" t="inlineStr">
+        <is>
+          <t>نعم</t>
+        </is>
+      </c>
+      <c r="H170" s="2" t="inlineStr">
+        <is>
+          <t>جرد + مراجعة</t>
+        </is>
+      </c>
+      <c r="I170" s="3" t="n">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="171">
+      <c r="A171" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="B171" s="2" t="inlineStr">
+        <is>
+          <t>الأربعاء</t>
+        </is>
+      </c>
+      <c r="C171" s="2" t="inlineStr">
+        <is>
+          <t>الرياض</t>
+        </is>
+      </c>
+      <c r="D171" s="2" t="n">
+        <v>58</v>
+      </c>
+      <c r="E171" s="2" t="inlineStr">
+        <is>
+          <t>د. حسام شلش</t>
+        </is>
+      </c>
+      <c r="F171" s="2" t="inlineStr"/>
+      <c r="G171" s="2" t="inlineStr">
+        <is>
+          <t>نعم</t>
+        </is>
+      </c>
+      <c r="H171" s="2" t="inlineStr">
+        <is>
+          <t>مراجعة فقط</t>
+        </is>
+      </c>
+      <c r="I171" s="3" t="n">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="172">
+      <c r="A172" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="B172" s="2" t="inlineStr">
+        <is>
+          <t>الأربعاء</t>
+        </is>
+      </c>
+      <c r="C172" s="2" t="inlineStr">
+        <is>
+          <t>الرياض</t>
+        </is>
+      </c>
+      <c r="D172" s="2" t="n">
+        <v>58</v>
+      </c>
+      <c r="E172" s="2" t="inlineStr">
+        <is>
+          <t>د. السيد حسن</t>
+        </is>
+      </c>
+      <c r="F172" s="2" t="inlineStr"/>
+      <c r="G172" s="2" t="inlineStr">
+        <is>
+          <t>نعم</t>
+        </is>
+      </c>
+      <c r="H172" s="2" t="inlineStr">
+        <is>
+          <t>مراجعة فقط</t>
+        </is>
+      </c>
+      <c r="I172" s="3" t="n">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="173">
+      <c r="A173" s="4" t="inlineStr">
         <is>
           <t>الإجمالي</t>
         </is>
       </c>
-      <c r="B167" s="4" t="n"/>
-      <c r="C167" s="4" t="n"/>
-      <c r="D167" s="4" t="n"/>
-      <c r="E167" s="4" t="n"/>
-      <c r="F167" s="4" t="n"/>
-      <c r="G167" s="4" t="n"/>
-      <c r="H167" s="4" t="n"/>
-      <c r="I167" s="5">
-        <f>SUM(I2:I166)</f>
-        <v>26950</v>
+      <c r="B173" s="4" t="n"/>
+      <c r="C173" s="4" t="n"/>
+      <c r="D173" s="4" t="n"/>
+      <c r="E173" s="4" t="n"/>
+      <c r="F173" s="4" t="n"/>
+      <c r="G173" s="4" t="n"/>
+      <c r="H173" s="4" t="n"/>
+      <c r="I173" s="5">
+        <f>SUM(I2:I172)</f>
+        <v>27950</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:I166"/>
+  <autoFilter ref="A1:I172"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Log Oct 22 counts (6, 13) and reviews for pharmacy 13; pharmacy 6 review pending
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01RnF4y3zxCG7NcjFkMnYdwu
</commit_message>
<xml_diff>
--- a/inventory/jard_log.xlsx
+++ b/inventory/jard_log.xlsx
@@ -10,7 +10,7 @@
     <sheet name="السجل" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'السجل'!$A$1:$I$172</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'السجل'!$A$1:$I$176</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -468,7 +468,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I173"/>
+  <dimension ref="A1:I177"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -7383,25 +7383,185 @@
       </c>
     </row>
     <row r="173">
-      <c r="A173" s="4" t="inlineStr">
+      <c r="A173" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-22</t>
+        </is>
+      </c>
+      <c r="B173" s="2" t="inlineStr">
+        <is>
+          <t>الخميس</t>
+        </is>
+      </c>
+      <c r="C173" s="2" t="inlineStr">
+        <is>
+          <t>الخرج</t>
+        </is>
+      </c>
+      <c r="D173" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="E173" s="2" t="inlineStr">
+        <is>
+          <t>د. حسام شلش</t>
+        </is>
+      </c>
+      <c r="F173" s="2" t="inlineStr">
+        <is>
+          <t>نعم</t>
+        </is>
+      </c>
+      <c r="G173" s="2" t="inlineStr"/>
+      <c r="H173" s="2" t="inlineStr">
+        <is>
+          <t>جرد فقط</t>
+        </is>
+      </c>
+      <c r="I173" s="3" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="174">
+      <c r="A174" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-22</t>
+        </is>
+      </c>
+      <c r="B174" s="2" t="inlineStr">
+        <is>
+          <t>الخميس</t>
+        </is>
+      </c>
+      <c r="C174" s="2" t="inlineStr">
+        <is>
+          <t>الخرج</t>
+        </is>
+      </c>
+      <c r="D174" s="2" t="n">
+        <v>13</v>
+      </c>
+      <c r="E174" s="2" t="inlineStr">
+        <is>
+          <t>د. حسام شلش</t>
+        </is>
+      </c>
+      <c r="F174" s="2" t="inlineStr">
+        <is>
+          <t>نعم</t>
+        </is>
+      </c>
+      <c r="G174" s="2" t="inlineStr">
+        <is>
+          <t>نعم</t>
+        </is>
+      </c>
+      <c r="H174" s="2" t="inlineStr">
+        <is>
+          <t>جرد + مراجعة</t>
+        </is>
+      </c>
+      <c r="I174" s="3" t="n">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="175">
+      <c r="A175" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-22</t>
+        </is>
+      </c>
+      <c r="B175" s="2" t="inlineStr">
+        <is>
+          <t>الخميس</t>
+        </is>
+      </c>
+      <c r="C175" s="2" t="inlineStr">
+        <is>
+          <t>الخرج</t>
+        </is>
+      </c>
+      <c r="D175" s="2" t="n">
+        <v>13</v>
+      </c>
+      <c r="E175" s="2" t="inlineStr">
+        <is>
+          <t>د. السيد حسن</t>
+        </is>
+      </c>
+      <c r="F175" s="2" t="inlineStr"/>
+      <c r="G175" s="2" t="inlineStr">
+        <is>
+          <t>نعم</t>
+        </is>
+      </c>
+      <c r="H175" s="2" t="inlineStr">
+        <is>
+          <t>مراجعة فقط</t>
+        </is>
+      </c>
+      <c r="I175" s="3" t="n">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="176">
+      <c r="A176" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-22</t>
+        </is>
+      </c>
+      <c r="B176" s="2" t="inlineStr">
+        <is>
+          <t>الخميس</t>
+        </is>
+      </c>
+      <c r="C176" s="2" t="inlineStr">
+        <is>
+          <t>الخرج</t>
+        </is>
+      </c>
+      <c r="D176" s="2" t="n">
+        <v>13</v>
+      </c>
+      <c r="E176" s="2" t="inlineStr">
+        <is>
+          <t>د. علي خليفة</t>
+        </is>
+      </c>
+      <c r="F176" s="2" t="inlineStr"/>
+      <c r="G176" s="2" t="inlineStr">
+        <is>
+          <t>نعم</t>
+        </is>
+      </c>
+      <c r="H176" s="2" t="inlineStr">
+        <is>
+          <t>مراجعة فقط</t>
+        </is>
+      </c>
+      <c r="I176" s="3" t="n">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="177">
+      <c r="A177" s="4" t="inlineStr">
         <is>
           <t>الإجمالي</t>
         </is>
       </c>
-      <c r="B173" s="4" t="n"/>
-      <c r="C173" s="4" t="n"/>
-      <c r="D173" s="4" t="n"/>
-      <c r="E173" s="4" t="n"/>
-      <c r="F173" s="4" t="n"/>
-      <c r="G173" s="4" t="n"/>
-      <c r="H173" s="4" t="n"/>
-      <c r="I173" s="5">
-        <f>SUM(I2:I172)</f>
-        <v>27950</v>
+      <c r="B177" s="4" t="n"/>
+      <c r="C177" s="4" t="n"/>
+      <c r="D177" s="4" t="n"/>
+      <c r="E177" s="4" t="n"/>
+      <c r="F177" s="4" t="n"/>
+      <c r="G177" s="4" t="n"/>
+      <c r="H177" s="4" t="n"/>
+      <c r="I177" s="5">
+        <f>SUM(I2:I176)</f>
+        <v>28550</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:I172"/>
+  <autoFilter ref="A1:I176"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Log Oct 22 reviews for pharmacy 6
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01RnF4y3zxCG7NcjFkMnYdwu
</commit_message>
<xml_diff>
--- a/inventory/jard_log.xlsx
+++ b/inventory/jard_log.xlsx
@@ -10,7 +10,7 @@
     <sheet name="السجل" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'السجل'!$A$1:$I$176</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'السجل'!$A$1:$I$177</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -468,7 +468,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I177"/>
+  <dimension ref="A1:I178"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -7411,14 +7411,18 @@
           <t>نعم</t>
         </is>
       </c>
-      <c r="G173" s="2" t="inlineStr"/>
+      <c r="G173" s="2" t="inlineStr">
+        <is>
+          <t>نعم</t>
+        </is>
+      </c>
       <c r="H173" s="2" t="inlineStr">
         <is>
-          <t>جرد فقط</t>
+          <t>جرد + مراجعة</t>
         </is>
       </c>
       <c r="I173" s="3" t="n">
-        <v>100</v>
+        <v>200</v>
       </c>
     </row>
     <row r="174">
@@ -7438,18 +7442,14 @@
         </is>
       </c>
       <c r="D174" s="2" t="n">
-        <v>13</v>
+        <v>6</v>
       </c>
       <c r="E174" s="2" t="inlineStr">
         <is>
-          <t>د. حسام شلش</t>
-        </is>
-      </c>
-      <c r="F174" s="2" t="inlineStr">
-        <is>
-          <t>نعم</t>
-        </is>
-      </c>
+          <t>د. علي خليفة</t>
+        </is>
+      </c>
+      <c r="F174" s="2" t="inlineStr"/>
       <c r="G174" s="2" t="inlineStr">
         <is>
           <t>نعم</t>
@@ -7457,11 +7457,11 @@
       </c>
       <c r="H174" s="2" t="inlineStr">
         <is>
-          <t>جرد + مراجعة</t>
+          <t>مراجعة فقط</t>
         </is>
       </c>
       <c r="I174" s="3" t="n">
-        <v>200</v>
+        <v>150</v>
       </c>
     </row>
     <row r="175">
@@ -7485,10 +7485,14 @@
       </c>
       <c r="E175" s="2" t="inlineStr">
         <is>
-          <t>د. السيد حسن</t>
-        </is>
-      </c>
-      <c r="F175" s="2" t="inlineStr"/>
+          <t>د. حسام شلش</t>
+        </is>
+      </c>
+      <c r="F175" s="2" t="inlineStr">
+        <is>
+          <t>نعم</t>
+        </is>
+      </c>
       <c r="G175" s="2" t="inlineStr">
         <is>
           <t>نعم</t>
@@ -7496,11 +7500,11 @@
       </c>
       <c r="H175" s="2" t="inlineStr">
         <is>
-          <t>مراجعة فقط</t>
+          <t>جرد + مراجعة</t>
         </is>
       </c>
       <c r="I175" s="3" t="n">
-        <v>150</v>
+        <v>200</v>
       </c>
     </row>
     <row r="176">
@@ -7524,7 +7528,7 @@
       </c>
       <c r="E176" s="2" t="inlineStr">
         <is>
-          <t>د. علي خليفة</t>
+          <t>د. السيد حسن</t>
         </is>
       </c>
       <c r="F176" s="2" t="inlineStr"/>
@@ -7543,25 +7547,64 @@
       </c>
     </row>
     <row r="177">
-      <c r="A177" s="4" t="inlineStr">
+      <c r="A177" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-22</t>
+        </is>
+      </c>
+      <c r="B177" s="2" t="inlineStr">
+        <is>
+          <t>الخميس</t>
+        </is>
+      </c>
+      <c r="C177" s="2" t="inlineStr">
+        <is>
+          <t>الخرج</t>
+        </is>
+      </c>
+      <c r="D177" s="2" t="n">
+        <v>13</v>
+      </c>
+      <c r="E177" s="2" t="inlineStr">
+        <is>
+          <t>د. علي خليفة</t>
+        </is>
+      </c>
+      <c r="F177" s="2" t="inlineStr"/>
+      <c r="G177" s="2" t="inlineStr">
+        <is>
+          <t>نعم</t>
+        </is>
+      </c>
+      <c r="H177" s="2" t="inlineStr">
+        <is>
+          <t>مراجعة فقط</t>
+        </is>
+      </c>
+      <c r="I177" s="3" t="n">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="178">
+      <c r="A178" s="4" t="inlineStr">
         <is>
           <t>الإجمالي</t>
         </is>
       </c>
-      <c r="B177" s="4" t="n"/>
-      <c r="C177" s="4" t="n"/>
-      <c r="D177" s="4" t="n"/>
-      <c r="E177" s="4" t="n"/>
-      <c r="F177" s="4" t="n"/>
-      <c r="G177" s="4" t="n"/>
-      <c r="H177" s="4" t="n"/>
-      <c r="I177" s="5">
-        <f>SUM(I2:I176)</f>
-        <v>28550</v>
+      <c r="B178" s="4" t="n"/>
+      <c r="C178" s="4" t="n"/>
+      <c r="D178" s="4" t="n"/>
+      <c r="E178" s="4" t="n"/>
+      <c r="F178" s="4" t="n"/>
+      <c r="G178" s="4" t="n"/>
+      <c r="H178" s="4" t="n"/>
+      <c r="I178" s="5">
+        <f>SUM(I2:I177)</f>
+        <v>28800</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:I176"/>
+  <autoFilter ref="A1:I177"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>